<commit_message>
Front End Data Comparison Add Device changes
</commit_message>
<xml_diff>
--- a/ExcelFiles/PatientSummary.xlsx
+++ b/ExcelFiles/PatientSummary.xlsx
@@ -8,67 +8,70 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Riomed\Cellma4ClinicalAuto\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ACD5EA1-6ECF-4927-98D2-11A9A21298F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{629DB74F-759A-44B0-86FB-8B18F7CF8C2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14660" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14660" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loginDetails" sheetId="2" r:id="rId1"/>
     <sheet name="PatientDetails" sheetId="3" r:id="rId2"/>
-    <sheet name="MedicationCategory" sheetId="1" r:id="rId3"/>
-    <sheet name="AddMedication" sheetId="4" r:id="rId4"/>
-    <sheet name="EditMedication" sheetId="6" r:id="rId5"/>
-    <sheet name="DeleteMedication" sheetId="22" r:id="rId6"/>
-    <sheet name="MedicationEDS" sheetId="5" r:id="rId7"/>
-    <sheet name="AddExamination" sheetId="7" r:id="rId8"/>
-    <sheet name="EditExamination" sheetId="8" r:id="rId9"/>
-    <sheet name="DeleteExamination" sheetId="10" r:id="rId10"/>
-    <sheet name="AddRecommendations" sheetId="9" r:id="rId11"/>
-    <sheet name="EditRecommendations" sheetId="17" r:id="rId12"/>
-    <sheet name="DeleteRecommendations" sheetId="18" r:id="rId13"/>
-    <sheet name="AddOutcome" sheetId="12" r:id="rId14"/>
-    <sheet name="EditOutcome" sheetId="13" r:id="rId15"/>
-    <sheet name="DeleteOutcome" sheetId="14" r:id="rId16"/>
-    <sheet name="AddDiagnosis" sheetId="11" r:id="rId17"/>
-    <sheet name="EditDiagnosis" sheetId="15" r:id="rId18"/>
-    <sheet name="DeleteDiagnosis" sheetId="16" r:id="rId19"/>
-    <sheet name="AddInterpretation" sheetId="19" r:id="rId20"/>
-    <sheet name="EditInterpretation" sheetId="20" r:id="rId21"/>
-    <sheet name="DeleteInterpretation" sheetId="21" r:id="rId22"/>
-    <sheet name="AddAllergy" sheetId="23" r:id="rId23"/>
-    <sheet name="EditAllergy" sheetId="24" r:id="rId24"/>
-    <sheet name="DeleteAllergy" sheetId="25" r:id="rId25"/>
-    <sheet name="AddProcedure" sheetId="26" r:id="rId26"/>
-    <sheet name="EditProcedure" sheetId="27" r:id="rId27"/>
-    <sheet name="DeleteProcedure" sheetId="28" r:id="rId28"/>
-    <sheet name="AddPatientScan" sheetId="29" r:id="rId29"/>
-    <sheet name="EditPatientScan" sheetId="30" r:id="rId30"/>
-    <sheet name="DeletePatientScan" sheetId="31" r:id="rId31"/>
-    <sheet name="AddProblems" sheetId="32" r:id="rId32"/>
-    <sheet name="EditProblems" sheetId="33" r:id="rId33"/>
-    <sheet name="DeleteProblems" sheetId="34" r:id="rId34"/>
-    <sheet name="AddOverview" sheetId="35" r:id="rId35"/>
-    <sheet name="EditOverview" sheetId="36" r:id="rId36"/>
-    <sheet name="DeleteOverview" sheetId="37" r:id="rId37"/>
-    <sheet name="Addsocial" sheetId="38" r:id="rId38"/>
-    <sheet name="Editsocial" sheetId="39" r:id="rId39"/>
-    <sheet name="Deletesocial" sheetId="40" r:id="rId40"/>
-    <sheet name="AddRiskFactor" sheetId="41" r:id="rId41"/>
-    <sheet name="EditRiskFactor" sheetId="42" r:id="rId42"/>
-    <sheet name="DeleteRiskFactor" sheetId="43" r:id="rId43"/>
-    <sheet name="AddLifestyle" sheetId="44" r:id="rId44"/>
-    <sheet name="EditLifestyle" sheetId="45" r:id="rId45"/>
-    <sheet name="DeleteLifestyle" sheetId="46" r:id="rId46"/>
-    <sheet name="AddInvestigation" sheetId="47" r:id="rId47"/>
-    <sheet name="EditInvestigation" sheetId="48" r:id="rId48"/>
-    <sheet name="AddCondition" sheetId="49" r:id="rId49"/>
-    <sheet name="EditCondition" sheetId="50" r:id="rId50"/>
-    <sheet name="DeleteCondition" sheetId="51" r:id="rId51"/>
-    <sheet name="AddPatientDetails" sheetId="52" r:id="rId52"/>
-    <sheet name="EditPatientDetails" sheetId="53" r:id="rId53"/>
-    <sheet name="DeletePatientDetails" sheetId="54" r:id="rId54"/>
-    <sheet name="AddTask" sheetId="55" r:id="rId55"/>
-    <sheet name="EditTask" sheetId="56" r:id="rId56"/>
+    <sheet name="DevicePatientDetails" sheetId="57" r:id="rId3"/>
+    <sheet name="AddDevice" sheetId="58" r:id="rId4"/>
+    <sheet name="EditDevice" sheetId="59" r:id="rId5"/>
+    <sheet name="MedicationCategory" sheetId="1" r:id="rId6"/>
+    <sheet name="AddMedication" sheetId="4" r:id="rId7"/>
+    <sheet name="EditMedication" sheetId="6" r:id="rId8"/>
+    <sheet name="DeleteMedication" sheetId="22" r:id="rId9"/>
+    <sheet name="MedicationEDS" sheetId="5" r:id="rId10"/>
+    <sheet name="AddExamination" sheetId="7" r:id="rId11"/>
+    <sheet name="EditExamination" sheetId="8" r:id="rId12"/>
+    <sheet name="DeleteExamination" sheetId="10" r:id="rId13"/>
+    <sheet name="AddRecommendations" sheetId="9" r:id="rId14"/>
+    <sheet name="EditRecommendations" sheetId="17" r:id="rId15"/>
+    <sheet name="DeleteRecommendations" sheetId="18" r:id="rId16"/>
+    <sheet name="AddOutcome" sheetId="12" r:id="rId17"/>
+    <sheet name="EditOutcome" sheetId="13" r:id="rId18"/>
+    <sheet name="DeleteOutcome" sheetId="14" r:id="rId19"/>
+    <sheet name="AddDiagnosis" sheetId="11" r:id="rId20"/>
+    <sheet name="EditDiagnosis" sheetId="15" r:id="rId21"/>
+    <sheet name="DeleteDiagnosis" sheetId="16" r:id="rId22"/>
+    <sheet name="AddInterpretation" sheetId="19" r:id="rId23"/>
+    <sheet name="EditInterpretation" sheetId="20" r:id="rId24"/>
+    <sheet name="DeleteInterpretation" sheetId="21" r:id="rId25"/>
+    <sheet name="AddAllergy" sheetId="23" r:id="rId26"/>
+    <sheet name="EditAllergy" sheetId="24" r:id="rId27"/>
+    <sheet name="DeleteAllergy" sheetId="25" r:id="rId28"/>
+    <sheet name="AddProcedure" sheetId="26" r:id="rId29"/>
+    <sheet name="EditProcedure" sheetId="27" r:id="rId30"/>
+    <sheet name="DeleteProcedure" sheetId="28" r:id="rId31"/>
+    <sheet name="AddPatientScan" sheetId="29" r:id="rId32"/>
+    <sheet name="EditPatientScan" sheetId="30" r:id="rId33"/>
+    <sheet name="DeletePatientScan" sheetId="31" r:id="rId34"/>
+    <sheet name="AddProblems" sheetId="32" r:id="rId35"/>
+    <sheet name="EditProblems" sheetId="33" r:id="rId36"/>
+    <sheet name="DeleteProblems" sheetId="34" r:id="rId37"/>
+    <sheet name="AddOverview" sheetId="35" r:id="rId38"/>
+    <sheet name="EditOverview" sheetId="36" r:id="rId39"/>
+    <sheet name="DeleteOverview" sheetId="37" r:id="rId40"/>
+    <sheet name="Addsocial" sheetId="38" r:id="rId41"/>
+    <sheet name="Editsocial" sheetId="39" r:id="rId42"/>
+    <sheet name="Deletesocial" sheetId="40" r:id="rId43"/>
+    <sheet name="AddRiskFactor" sheetId="41" r:id="rId44"/>
+    <sheet name="EditRiskFactor" sheetId="42" r:id="rId45"/>
+    <sheet name="DeleteRiskFactor" sheetId="43" r:id="rId46"/>
+    <sheet name="AddLifestyle" sheetId="44" r:id="rId47"/>
+    <sheet name="EditLifestyle" sheetId="45" r:id="rId48"/>
+    <sheet name="DeleteLifestyle" sheetId="46" r:id="rId49"/>
+    <sheet name="AddInvestigation" sheetId="47" r:id="rId50"/>
+    <sheet name="EditInvestigation" sheetId="48" r:id="rId51"/>
+    <sheet name="AddCondition" sheetId="49" r:id="rId52"/>
+    <sheet name="EditCondition" sheetId="50" r:id="rId53"/>
+    <sheet name="DeleteCondition" sheetId="51" r:id="rId54"/>
+    <sheet name="AddPatientDetails" sheetId="52" r:id="rId55"/>
+    <sheet name="EditPatientDetails" sheetId="53" r:id="rId56"/>
+    <sheet name="DeletePatientDetails" sheetId="54" r:id="rId57"/>
+    <sheet name="AddTask" sheetId="55" r:id="rId58"/>
+    <sheet name="EditTask" sheetId="56" r:id="rId59"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -91,7 +94,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="833" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="891" uniqueCount="426">
   <si>
     <t>username</t>
   </si>
@@ -1267,6 +1270,108 @@
   </si>
   <si>
     <t>given</t>
+  </si>
+  <si>
+    <t>AkaliA</t>
+  </si>
+  <si>
+    <t>Riomedtest</t>
+  </si>
+  <si>
+    <t>08/09/2024</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Cochlear Osia OSI200</t>
+  </si>
+  <si>
+    <t>dev_name</t>
+  </si>
+  <si>
+    <t>dev_type</t>
+  </si>
+  <si>
+    <t>Device</t>
+  </si>
+  <si>
+    <t>dev_procedure_name</t>
+  </si>
+  <si>
+    <t>Cochlear Implantation</t>
+  </si>
+  <si>
+    <t>dev_manufacturer</t>
+  </si>
+  <si>
+    <t>Cochlear</t>
+  </si>
+  <si>
+    <t>dev_deleted_reason</t>
+  </si>
+  <si>
+    <t>Device deleted</t>
+  </si>
+  <si>
+    <t>dev_expiry_date</t>
+  </si>
+  <si>
+    <t>ded_type</t>
+  </si>
+  <si>
+    <t>ded_internal_external</t>
+  </si>
+  <si>
+    <t>ded_laterality</t>
+  </si>
+  <si>
+    <t>ded_notes</t>
+  </si>
+  <si>
+    <t>Device added</t>
+  </si>
+  <si>
+    <t>ded_status</t>
+  </si>
+  <si>
+    <t>Tool</t>
+  </si>
+  <si>
+    <t>SA Company</t>
+  </si>
+  <si>
+    <t>Device edited</t>
+  </si>
+  <si>
+    <t>28/02/2025</t>
+  </si>
+  <si>
+    <t>ded_type_entry</t>
+  </si>
+  <si>
+    <t>ded_internal_external_entry</t>
+  </si>
+  <si>
+    <t>Internal</t>
+  </si>
+  <si>
+    <t>ded_laterality_entry</t>
+  </si>
+  <si>
+    <t>ded_status_entry</t>
+  </si>
+  <si>
+    <t>External</t>
+  </si>
+  <si>
+    <t>Issued</t>
+  </si>
+  <si>
+    <t>First Stage</t>
+  </si>
+  <si>
+    <t>31/03/2025</t>
   </si>
 </sst>
 </file>
@@ -1674,6 +1779,155 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3310FF1D-4559-4E35-BB7B-0285AF82C887}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82EC7FC3-A185-46F7-A2D4-55C9E247ADD9}">
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="2" width="23.81640625" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" customWidth="1"/>
+    <col min="4" max="4" width="22.26953125" customWidth="1"/>
+    <col min="5" max="5" width="17.453125" customWidth="1"/>
+    <col min="6" max="6" width="15.1796875" customWidth="1"/>
+    <col min="7" max="7" width="17.54296875" customWidth="1"/>
+    <col min="8" max="8" width="16.54296875" customWidth="1"/>
+    <col min="9" max="9" width="26.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>226</v>
+      </c>
+      <c r="C1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F1" t="s">
+        <v>136</v>
+      </c>
+      <c r="G1" t="s">
+        <v>121</v>
+      </c>
+      <c r="H1" t="s">
+        <v>130</v>
+      </c>
+      <c r="I1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="18.75" customHeight="1">
+      <c r="A2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D2" t="s">
+        <v>129</v>
+      </c>
+      <c r="E2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F2" s="8">
+        <v>45407</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="H2" t="s">
+        <v>131</v>
+      </c>
+      <c r="I2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{538BA7B8-E3A5-4977-A6D8-AD18062987D5}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.453125" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" customWidth="1"/>
+    <col min="4" max="4" width="14.453125" customWidth="1"/>
+    <col min="5" max="5" width="16.453125" customWidth="1"/>
+    <col min="6" max="6" width="15.26953125" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>128</v>
+      </c>
+      <c r="D1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="18.75" customHeight="1">
+      <c r="A2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D2" t="s">
+        <v>135</v>
+      </c>
+      <c r="E2" s="8">
+        <v>45407</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5682E5CD-63B5-4779-9930-5C9E9312DCA8}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -1703,7 +1957,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7070D364-07A9-4E81-9AAD-6D06CFE64A7E}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -1761,7 +2015,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4C74051-56F8-4BE3-95DE-85BE5950FD64}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -1811,7 +2065,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69EDCE76-70F4-4473-B92F-8913C9A903B8}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -1847,7 +2101,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F50D2E72-168F-40F2-B5D3-65D8E679AC63}">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -1923,7 +2177,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8027F072-5B7F-474B-8D83-79953C31361B}">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -2002,7 +2256,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{008CC7AC-AB6D-4187-B6A0-1158E613B828}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -2032,7 +2286,257 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFF0DF87-67F2-4E87-A7EE-C4365800D834}">
+  <dimension ref="A1:AV2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="2" max="2" width="18.26953125" customWidth="1"/>
+    <col min="7" max="7" width="16.453125" customWidth="1"/>
+    <col min="9" max="9" width="11.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:48" s="2" customFormat="1">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" t="s">
+        <v>16</v>
+      </c>
+      <c r="N1" t="s">
+        <v>17</v>
+      </c>
+      <c r="O1" t="s">
+        <v>18</v>
+      </c>
+      <c r="P1" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>20</v>
+      </c>
+      <c r="R1" t="s">
+        <v>21</v>
+      </c>
+      <c r="S1" t="s">
+        <v>22</v>
+      </c>
+      <c r="T1" t="s">
+        <v>23</v>
+      </c>
+      <c r="U1" t="s">
+        <v>24</v>
+      </c>
+      <c r="V1" t="s">
+        <v>25</v>
+      </c>
+      <c r="W1" t="s">
+        <v>26</v>
+      </c>
+      <c r="X1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AS1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>50</v>
+      </c>
+      <c r="AV1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:48" s="2" customFormat="1" ht="43.5">
+      <c r="B2" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="W2" s="2">
+        <v>0</v>
+      </c>
+      <c r="X2" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="Y2" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z2" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="AB2" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="AI2" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="AJ2" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AM2" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AO2" t="s">
+        <v>62</v>
+      </c>
+      <c r="AQ2" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="AR2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AU2" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="AV2" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{094FA7C7-2F9F-473D-A811-B803747DC0A3}">
   <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -2138,7 +2642,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92D95DB8-7522-4276-90BD-0BAB60F0AAE6}">
   <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -2231,7 +2735,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70DCF4C9-25DB-44CD-A95D-99E79260CBAB}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -2261,257 +2765,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFF0DF87-67F2-4E87-A7EE-C4365800D834}">
-  <dimension ref="A1:AV2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="2" max="2" width="18.26953125" customWidth="1"/>
-    <col min="7" max="7" width="16.453125" customWidth="1"/>
-    <col min="9" max="9" width="11.1796875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:48" s="2" customFormat="1">
-      <c r="A1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I1" t="s">
-        <v>12</v>
-      </c>
-      <c r="J1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K1" t="s">
-        <v>14</v>
-      </c>
-      <c r="L1" t="s">
-        <v>15</v>
-      </c>
-      <c r="M1" t="s">
-        <v>16</v>
-      </c>
-      <c r="N1" t="s">
-        <v>17</v>
-      </c>
-      <c r="O1" t="s">
-        <v>18</v>
-      </c>
-      <c r="P1" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>20</v>
-      </c>
-      <c r="R1" t="s">
-        <v>21</v>
-      </c>
-      <c r="S1" t="s">
-        <v>22</v>
-      </c>
-      <c r="T1" t="s">
-        <v>23</v>
-      </c>
-      <c r="U1" t="s">
-        <v>24</v>
-      </c>
-      <c r="V1" t="s">
-        <v>25</v>
-      </c>
-      <c r="W1" t="s">
-        <v>26</v>
-      </c>
-      <c r="X1" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>29</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>31</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>32</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>34</v>
-      </c>
-      <c r="AF1" t="s">
-        <v>35</v>
-      </c>
-      <c r="AG1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AH1" t="s">
-        <v>37</v>
-      </c>
-      <c r="AI1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AJ1" t="s">
-        <v>39</v>
-      </c>
-      <c r="AK1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AL1" t="s">
-        <v>41</v>
-      </c>
-      <c r="AM1" t="s">
-        <v>42</v>
-      </c>
-      <c r="AN1" t="s">
-        <v>43</v>
-      </c>
-      <c r="AO1" t="s">
-        <v>44</v>
-      </c>
-      <c r="AP1" t="s">
-        <v>45</v>
-      </c>
-      <c r="AQ1" t="s">
-        <v>46</v>
-      </c>
-      <c r="AR1" t="s">
-        <v>47</v>
-      </c>
-      <c r="AS1" t="s">
-        <v>48</v>
-      </c>
-      <c r="AT1" t="s">
-        <v>49</v>
-      </c>
-      <c r="AU1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AV1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="2" spans="1:48" s="2" customFormat="1" ht="43.5">
-      <c r="B2" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>278</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="S2" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="U2" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="V2" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="W2" s="2">
-        <v>0</v>
-      </c>
-      <c r="X2" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="Y2" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z2" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="AB2" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="AI2" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="AJ2" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AM2" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="AO2" t="s">
-        <v>62</v>
-      </c>
-      <c r="AQ2" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="AR2" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AU2" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="AV2" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{073326C8-FACB-4B5B-B1CF-ABFED8B93DBE}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -2569,7 +2823,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F596452A-5694-4E32-87F2-C18569884D3B}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -2627,7 +2881,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8852AC2C-7F1F-45E0-AA81-1C0AC8298BDB}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -2664,7 +2918,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C664057-036F-45F9-BB17-F131467544E4}">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -2718,7 +2972,7 @@
       </c>
       <c r="D2" s="7">
         <f ca="1">TODAY()</f>
-        <v>45679</v>
+        <v>45698</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>206</v>
@@ -2739,7 +2993,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DE09E9A-9C0C-49EF-BEE4-12AF4C853339}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -2792,7 +3046,7 @@
       </c>
       <c r="D2" s="7">
         <f ca="1">TODAY()</f>
-        <v>45679</v>
+        <v>45698</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>207</v>
@@ -2812,7 +3066,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F4129C8-341D-4D38-92A2-748311EBE13A}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -2849,7 +3103,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9AC72BC-1449-4578-8E57-945920649F3D}">
   <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -2921,11 +3175,11 @@
       </c>
       <c r="C2" s="8">
         <f ca="1">TODAY()</f>
-        <v>45679</v>
+        <v>45698</v>
       </c>
       <c r="D2" s="11" t="str">
         <f ca="1">TEXT(C2, "DD-MM-YYYY")</f>
-        <v>22-01-2025</v>
+        <v>10-02-2025</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>106</v>
@@ -2963,7 +3217,51 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7AEB4A7-C8C6-4BF4-A6C6-FFEA2B919D62}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.453125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>394</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80A773DA-484D-48A0-B5A2-743931447EDE}">
   <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -3025,7 +3323,7 @@
       </c>
       <c r="C2" s="7">
         <f ca="1">TODAY()</f>
-        <v>45679</v>
+        <v>45698</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>106</v>
@@ -3060,7 +3358,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3A63575-EEB1-470D-A815-33D356B026F2}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -3097,7 +3395,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A6156A5-E27D-4C56-9CFB-F9306D57D7B5}">
   <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -3192,16 +3490,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DDECB00-706E-4E8F-A123-3F48B34B46C2}">
   <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -3308,7 +3597,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAB902D2-410D-470A-9E88-FE4AC8B16D55}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -3338,7 +3627,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89AB0309-4D83-402B-A384-3BBD8F0E5F31}">
   <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -3431,7 +3720,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B38BF4A6-8DEB-41FA-A7FD-F0100AB3FE2C}">
   <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -3524,7 +3813,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC23809B-2D36-41E4-A3B9-65D4308A6DCA}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -3554,7 +3843,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FF9792A-063B-40AF-9553-C8061AFC39D0}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -3612,7 +3901,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B8717C7-2D4F-48DD-A7CA-84784DCBB919}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -3656,7 +3945,125 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73B66876-3BB3-48A1-BCF1-747C769152D0}">
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.90625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.453125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" t="s">
+        <v>397</v>
+      </c>
+      <c r="B1" t="s">
+        <v>398</v>
+      </c>
+      <c r="C1" t="s">
+        <v>400</v>
+      </c>
+      <c r="D1" t="s">
+        <v>402</v>
+      </c>
+      <c r="E1" t="s">
+        <v>406</v>
+      </c>
+      <c r="F1" t="s">
+        <v>407</v>
+      </c>
+      <c r="G1" t="s">
+        <v>417</v>
+      </c>
+      <c r="H1" t="s">
+        <v>408</v>
+      </c>
+      <c r="I1" t="s">
+        <v>418</v>
+      </c>
+      <c r="J1" t="s">
+        <v>409</v>
+      </c>
+      <c r="K1" t="s">
+        <v>420</v>
+      </c>
+      <c r="L1" t="s">
+        <v>410</v>
+      </c>
+      <c r="M1" t="s">
+        <v>412</v>
+      </c>
+      <c r="N1" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" t="s">
+        <v>396</v>
+      </c>
+      <c r="B2" t="s">
+        <v>399</v>
+      </c>
+      <c r="C2" t="s">
+        <v>401</v>
+      </c>
+      <c r="D2" t="s">
+        <v>403</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="F2" t="str">
+        <f>LOWER(G2)</f>
+        <v>primary</v>
+      </c>
+      <c r="G2" t="s">
+        <v>220</v>
+      </c>
+      <c r="H2" t="str">
+        <f>LOWER(I2)</f>
+        <v>internal</v>
+      </c>
+      <c r="I2" t="s">
+        <v>419</v>
+      </c>
+      <c r="J2" t="str">
+        <f>LOWER(K2)</f>
+        <v>left</v>
+      </c>
+      <c r="K2" t="s">
+        <v>106</v>
+      </c>
+      <c r="L2" t="s">
+        <v>411</v>
+      </c>
+      <c r="M2" t="str">
+        <f>LOWER(N2)</f>
+        <v>requested</v>
+      </c>
+      <c r="N2" t="s">
+        <v>215</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BF370ED-86AA-4D7E-B092-14AB12F95410}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -3686,7 +4093,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28DAC4B0-6F7A-40C4-8629-2F293F19EE6C}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -3730,7 +4137,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4EF1174-5299-4F4F-A888-C15D55804D2F}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -3774,7 +4181,1174 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF82F3D0-82CD-49AF-BA0A-7CEE53FBA6AC}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="28.1796875" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>280</v>
+      </c>
+      <c r="B2" t="s">
+        <v>273</v>
+      </c>
+      <c r="C2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFEABC41-711E-4537-AE0B-FD45295FCA16}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="19.26953125" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" customWidth="1"/>
+    <col min="4" max="4" width="22.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>284</v>
+      </c>
+      <c r="D1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="29">
+      <c r="A2" t="s">
+        <v>285</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="D2" t="s">
+        <v>282</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BCAE196-8758-4745-8A92-E19A1A017AF5}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="19.26953125" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" customWidth="1"/>
+    <col min="4" max="4" width="22.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>284</v>
+      </c>
+      <c r="D1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="29">
+      <c r="A2" t="s">
+        <v>285</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="D2" t="s">
+        <v>282</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA3F2689-A05C-47BB-9880-495021A0BDBF}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="28.1796875" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>281</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="C2" t="s">
+        <v>287</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{025D1112-B23A-48F4-BA89-51264C4515AC}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.26953125" customWidth="1"/>
+    <col min="3" max="4" width="16.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>289</v>
+      </c>
+      <c r="D1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="29">
+      <c r="A2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B2" t="s">
+        <v>387</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="D2" t="s">
+        <v>288</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD2F5B74-CFA6-4CF1-AE93-E1D942D7EC4C}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.26953125" customWidth="1"/>
+    <col min="3" max="4" width="16.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>289</v>
+      </c>
+      <c r="D1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="29">
+      <c r="A2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B2" t="s">
+        <v>387</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="D2" t="s">
+        <v>288</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{206A2E86-90FC-4080-A7DC-7A2B6DBA9D36}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="28.1796875" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B2" t="s">
+        <v>387</v>
+      </c>
+      <c r="C2" t="s">
+        <v>293</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7334FDE5-0DFC-4860-A6DD-AB90F5178C6D}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="24.90625" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="15.453125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15">
+      <c r="A1" t="s">
+        <v>397</v>
+      </c>
+      <c r="B1" t="s">
+        <v>398</v>
+      </c>
+      <c r="C1" t="s">
+        <v>400</v>
+      </c>
+      <c r="D1" t="s">
+        <v>402</v>
+      </c>
+      <c r="E1" t="s">
+        <v>404</v>
+      </c>
+      <c r="F1" t="s">
+        <v>406</v>
+      </c>
+      <c r="G1" t="s">
+        <v>407</v>
+      </c>
+      <c r="H1" t="s">
+        <v>417</v>
+      </c>
+      <c r="I1" t="s">
+        <v>408</v>
+      </c>
+      <c r="J1" t="s">
+        <v>418</v>
+      </c>
+      <c r="K1" t="s">
+        <v>409</v>
+      </c>
+      <c r="L1" t="s">
+        <v>420</v>
+      </c>
+      <c r="M1" t="s">
+        <v>410</v>
+      </c>
+      <c r="N1" t="s">
+        <v>412</v>
+      </c>
+      <c r="O1" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
+      <c r="A2" t="s">
+        <v>396</v>
+      </c>
+      <c r="B2" t="s">
+        <v>413</v>
+      </c>
+      <c r="C2" t="s">
+        <v>401</v>
+      </c>
+      <c r="D2" t="s">
+        <v>414</v>
+      </c>
+      <c r="E2" t="s">
+        <v>405</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>425</v>
+      </c>
+      <c r="G2" t="str">
+        <f>SUBSTITUTE(LOWER(H2)," ","")</f>
+        <v>firststage</v>
+      </c>
+      <c r="H2" t="s">
+        <v>424</v>
+      </c>
+      <c r="I2" t="str">
+        <f>LOWER(J2)</f>
+        <v>external</v>
+      </c>
+      <c r="J2" t="s">
+        <v>422</v>
+      </c>
+      <c r="K2" t="str">
+        <f>LOWER(L2)</f>
+        <v>right</v>
+      </c>
+      <c r="L2" t="s">
+        <v>193</v>
+      </c>
+      <c r="M2" t="s">
+        <v>415</v>
+      </c>
+      <c r="N2" t="str">
+        <f>LOWER(O2)</f>
+        <v>issued</v>
+      </c>
+      <c r="O2" t="s">
+        <v>423</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA6646E2-86C9-4AB0-83E3-F184F5C30E9A}">
+  <dimension ref="A1:Q2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="16.7265625" customWidth="1"/>
+    <col min="5" max="5" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.26953125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17">
+      <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>302</v>
+      </c>
+      <c r="D1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E1" t="s">
+        <v>303</v>
+      </c>
+      <c r="F1" t="s">
+        <v>304</v>
+      </c>
+      <c r="G1" t="s">
+        <v>305</v>
+      </c>
+      <c r="H1" t="s">
+        <v>306</v>
+      </c>
+      <c r="I1" t="s">
+        <v>307</v>
+      </c>
+      <c r="J1" t="s">
+        <v>308</v>
+      </c>
+      <c r="K1" t="s">
+        <v>309</v>
+      </c>
+      <c r="L1" t="s">
+        <v>310</v>
+      </c>
+      <c r="M1" t="s">
+        <v>311</v>
+      </c>
+      <c r="N1" t="s">
+        <v>312</v>
+      </c>
+      <c r="O1" t="s">
+        <v>313</v>
+      </c>
+      <c r="P1" t="s">
+        <v>314</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17">
+      <c r="A2" t="s">
+        <v>299</v>
+      </c>
+      <c r="B2" t="s">
+        <v>300</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D2" t="s">
+        <v>301</v>
+      </c>
+      <c r="F2" t="s">
+        <v>324</v>
+      </c>
+      <c r="G2" t="s">
+        <v>323</v>
+      </c>
+      <c r="H2" t="s">
+        <v>135</v>
+      </c>
+      <c r="I2" t="s">
+        <v>103</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="K2" t="s">
+        <v>101</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>320</v>
+      </c>
+      <c r="N2" t="s">
+        <v>319</v>
+      </c>
+      <c r="O2" t="s">
+        <v>318</v>
+      </c>
+      <c r="P2" t="s">
+        <v>317</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>316</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{132C5A93-3712-47E8-A929-16017ECD465E}">
+  <dimension ref="A1:U2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="16.7265625" customWidth="1"/>
+    <col min="5" max="5" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="23" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:21">
+      <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>302</v>
+      </c>
+      <c r="D1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E1" t="s">
+        <v>303</v>
+      </c>
+      <c r="F1" t="s">
+        <v>304</v>
+      </c>
+      <c r="G1" t="s">
+        <v>305</v>
+      </c>
+      <c r="H1" t="s">
+        <v>306</v>
+      </c>
+      <c r="I1" t="s">
+        <v>307</v>
+      </c>
+      <c r="J1" t="s">
+        <v>308</v>
+      </c>
+      <c r="K1" t="s">
+        <v>309</v>
+      </c>
+      <c r="L1" t="s">
+        <v>310</v>
+      </c>
+      <c r="M1" t="s">
+        <v>311</v>
+      </c>
+      <c r="N1" t="s">
+        <v>312</v>
+      </c>
+      <c r="O1" t="s">
+        <v>313</v>
+      </c>
+      <c r="P1" t="s">
+        <v>314</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>315</v>
+      </c>
+      <c r="R1" t="s">
+        <v>328</v>
+      </c>
+      <c r="S1" t="s">
+        <v>329</v>
+      </c>
+      <c r="T1" t="s">
+        <v>330</v>
+      </c>
+      <c r="U1" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21">
+      <c r="A2" t="s">
+        <v>299</v>
+      </c>
+      <c r="B2" t="s">
+        <v>300</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="D2" t="s">
+        <v>301</v>
+      </c>
+      <c r="F2" t="s">
+        <v>324</v>
+      </c>
+      <c r="G2" t="s">
+        <v>326</v>
+      </c>
+      <c r="H2" t="s">
+        <v>135</v>
+      </c>
+      <c r="I2" t="s">
+        <v>103</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="K2" t="s">
+        <v>101</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>320</v>
+      </c>
+      <c r="N2" t="s">
+        <v>319</v>
+      </c>
+      <c r="O2" t="s">
+        <v>318</v>
+      </c>
+      <c r="P2" t="s">
+        <v>317</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>327</v>
+      </c>
+      <c r="R2" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="S2" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="T2" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="U2" s="6" t="s">
+        <v>333</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1194F774-EACE-44AC-9C8A-A1CC70FE36E1}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="2" max="3" width="25.54296875" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="19.26953125" customWidth="1"/>
+    <col min="6" max="6" width="14.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>334</v>
+      </c>
+      <c r="D1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E1" t="s">
+        <v>335</v>
+      </c>
+      <c r="F1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="18.75" customHeight="1">
+      <c r="A2" t="s">
+        <v>336</v>
+      </c>
+      <c r="B2" t="s">
+        <v>337</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="F2" t="s">
+        <v>341</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01C7CE86-1D30-42A6-BFFE-DD7CB531D10C}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="2" max="3" width="25.54296875" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="19.26953125" customWidth="1"/>
+    <col min="6" max="6" width="14.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>334</v>
+      </c>
+      <c r="D1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E1" t="s">
+        <v>335</v>
+      </c>
+      <c r="F1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="18.75" customHeight="1">
+      <c r="A2" t="s">
+        <v>336</v>
+      </c>
+      <c r="B2" t="s">
+        <v>337</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="F2" t="s">
+        <v>341</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06A0A6C0-CF2F-48B8-BAC5-F3E5690001A5}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="2" max="2" width="25.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>336</v>
+      </c>
+      <c r="B2" t="s">
+        <v>337</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{120AD279-3012-4840-AF87-588B2BE3B2AA}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>130</v>
+      </c>
+      <c r="D1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>345</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="C2" t="s">
+        <v>347</v>
+      </c>
+      <c r="D2" t="s">
+        <v>348</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C038ED2-3C9D-4D5B-A9F6-773661E9B6A6}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>130</v>
+      </c>
+      <c r="D1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>345</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="C2" t="s">
+        <v>347</v>
+      </c>
+      <c r="D2" t="s">
+        <v>348</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{796CA3FD-2DF2-4849-A599-7F2B1477C186}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>345</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>349</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C6C2239-2180-4B9C-B8A1-E16F3FCE77A5}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="14.26953125" customWidth="1"/>
+    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15">
+      <c r="A1" t="s">
+        <v>350</v>
+      </c>
+      <c r="B1" t="s">
+        <v>351</v>
+      </c>
+      <c r="C1" t="s">
+        <v>352</v>
+      </c>
+      <c r="D1" t="s">
+        <v>353</v>
+      </c>
+      <c r="E1" t="s">
+        <v>354</v>
+      </c>
+      <c r="F1" t="s">
+        <v>355</v>
+      </c>
+      <c r="G1" t="s">
+        <v>356</v>
+      </c>
+      <c r="H1" t="s">
+        <v>357</v>
+      </c>
+      <c r="I1" t="s">
+        <v>358</v>
+      </c>
+      <c r="J1" t="s">
+        <v>359</v>
+      </c>
+      <c r="K1" t="s">
+        <v>360</v>
+      </c>
+      <c r="L1" t="s">
+        <v>361</v>
+      </c>
+      <c r="M1" t="s">
+        <v>362</v>
+      </c>
+      <c r="N1" t="s">
+        <v>363</v>
+      </c>
+      <c r="O1" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
+      <c r="A2" t="s">
+        <v>365</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>366</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>367</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>368</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>369</v>
+      </c>
+      <c r="F2" t="s">
+        <v>370</v>
+      </c>
+      <c r="G2" t="s">
+        <v>383</v>
+      </c>
+      <c r="H2" t="s">
+        <v>101</v>
+      </c>
+      <c r="I2" t="s">
+        <v>371</v>
+      </c>
+      <c r="J2" t="s">
+        <v>372</v>
+      </c>
+      <c r="K2" t="s">
+        <v>373</v>
+      </c>
+      <c r="L2" t="s">
+        <v>374</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="N2" s="6" t="s">
+        <v>375</v>
+      </c>
+      <c r="O2" t="s">
+        <v>376</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B730A7AF-1268-4970-A808-63C4CFDE9D42}">
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" t="s">
+        <v>377</v>
+      </c>
+      <c r="B1" t="s">
+        <v>378</v>
+      </c>
+      <c r="C1" t="s">
+        <v>355</v>
+      </c>
+      <c r="D1" t="s">
+        <v>356</v>
+      </c>
+      <c r="E1" t="s">
+        <v>357</v>
+      </c>
+      <c r="F1" t="s">
+        <v>358</v>
+      </c>
+      <c r="G1" t="s">
+        <v>379</v>
+      </c>
+      <c r="H1" t="s">
+        <v>315</v>
+      </c>
+      <c r="I1" t="s">
+        <v>362</v>
+      </c>
+      <c r="J1" t="s">
+        <v>363</v>
+      </c>
+      <c r="K1" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>381</v>
+      </c>
+      <c r="C2" t="s">
+        <v>370</v>
+      </c>
+      <c r="D2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E2" t="s">
+        <v>101</v>
+      </c>
+      <c r="F2" t="s">
+        <v>371</v>
+      </c>
+      <c r="G2" t="s">
+        <v>373</v>
+      </c>
+      <c r="H2" t="s">
+        <v>382</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>375</v>
+      </c>
+      <c r="K2" t="s">
+        <v>376</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="18.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DD9439C-0973-45AC-88BC-21584AF7E144}">
   <dimension ref="A1:AG2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -4016,618 +5590,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF82F3D0-82CD-49AF-BA0A-7CEE53FBA6AC}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="28.1796875" customWidth="1"/>
-    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.453125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>280</v>
-      </c>
-      <c r="B2" t="s">
-        <v>273</v>
-      </c>
-      <c r="C2" t="s">
-        <v>127</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFEABC41-711E-4537-AE0B-FD45295FCA16}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="19.26953125" customWidth="1"/>
-    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.453125" customWidth="1"/>
-    <col min="4" max="4" width="22.1796875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C1" t="s">
-        <v>284</v>
-      </c>
-      <c r="D1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="29">
-      <c r="A2" t="s">
-        <v>285</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>343</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="D2" t="s">
-        <v>282</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BCAE196-8758-4745-8A92-E19A1A017AF5}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="19.26953125" customWidth="1"/>
-    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.453125" customWidth="1"/>
-    <col min="4" max="4" width="22.1796875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C1" t="s">
-        <v>284</v>
-      </c>
-      <c r="D1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="29">
-      <c r="A2" t="s">
-        <v>285</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>343</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>286</v>
-      </c>
-      <c r="D2" t="s">
-        <v>282</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA3F2689-A05C-47BB-9880-495021A0BDBF}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="28.1796875" customWidth="1"/>
-    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.453125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>281</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>343</v>
-      </c>
-      <c r="C2" t="s">
-        <v>287</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{025D1112-B23A-48F4-BA89-51264C4515AC}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.26953125" customWidth="1"/>
-    <col min="3" max="4" width="16.7265625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C1" t="s">
-        <v>289</v>
-      </c>
-      <c r="D1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="29">
-      <c r="A2" t="s">
-        <v>290</v>
-      </c>
-      <c r="B2" t="s">
-        <v>387</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="D2" t="s">
-        <v>288</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD2F5B74-CFA6-4CF1-AE93-E1D942D7EC4C}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.26953125" customWidth="1"/>
-    <col min="3" max="4" width="16.7265625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C1" t="s">
-        <v>289</v>
-      </c>
-      <c r="D1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="29">
-      <c r="A2" t="s">
-        <v>290</v>
-      </c>
-      <c r="B2" t="s">
-        <v>387</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>291</v>
-      </c>
-      <c r="D2" t="s">
-        <v>288</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{206A2E86-90FC-4080-A7DC-7A2B6DBA9D36}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="28.1796875" customWidth="1"/>
-    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.453125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>290</v>
-      </c>
-      <c r="B2" t="s">
-        <v>387</v>
-      </c>
-      <c r="C2" t="s">
-        <v>293</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA6646E2-86C9-4AB0-83E3-F184F5C30E9A}">
-  <dimension ref="A1:Q2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="16.7265625" customWidth="1"/>
-    <col min="5" max="5" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.26953125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:17">
-      <c r="A1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C1" t="s">
-        <v>302</v>
-      </c>
-      <c r="D1" t="s">
-        <v>130</v>
-      </c>
-      <c r="E1" t="s">
-        <v>303</v>
-      </c>
-      <c r="F1" t="s">
-        <v>304</v>
-      </c>
-      <c r="G1" t="s">
-        <v>305</v>
-      </c>
-      <c r="H1" t="s">
-        <v>306</v>
-      </c>
-      <c r="I1" t="s">
-        <v>307</v>
-      </c>
-      <c r="J1" t="s">
-        <v>308</v>
-      </c>
-      <c r="K1" t="s">
-        <v>309</v>
-      </c>
-      <c r="L1" t="s">
-        <v>310</v>
-      </c>
-      <c r="M1" t="s">
-        <v>311</v>
-      </c>
-      <c r="N1" t="s">
-        <v>312</v>
-      </c>
-      <c r="O1" t="s">
-        <v>313</v>
-      </c>
-      <c r="P1" t="s">
-        <v>314</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17">
-      <c r="A2" t="s">
-        <v>299</v>
-      </c>
-      <c r="B2" t="s">
-        <v>300</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="D2" t="s">
-        <v>301</v>
-      </c>
-      <c r="F2" t="s">
-        <v>324</v>
-      </c>
-      <c r="G2" t="s">
-        <v>323</v>
-      </c>
-      <c r="H2" t="s">
-        <v>135</v>
-      </c>
-      <c r="I2" t="s">
-        <v>103</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>322</v>
-      </c>
-      <c r="K2" t="s">
-        <v>101</v>
-      </c>
-      <c r="L2" s="6" t="s">
-        <v>321</v>
-      </c>
-      <c r="M2" s="6" t="s">
-        <v>320</v>
-      </c>
-      <c r="N2" t="s">
-        <v>319</v>
-      </c>
-      <c r="O2" t="s">
-        <v>318</v>
-      </c>
-      <c r="P2" t="s">
-        <v>317</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>316</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{132C5A93-3712-47E8-A929-16017ECD465E}">
-  <dimension ref="A1:U2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="16.7265625" customWidth="1"/>
-    <col min="5" max="5" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.26953125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="23" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:21">
-      <c r="A1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C1" t="s">
-        <v>302</v>
-      </c>
-      <c r="D1" t="s">
-        <v>130</v>
-      </c>
-      <c r="E1" t="s">
-        <v>303</v>
-      </c>
-      <c r="F1" t="s">
-        <v>304</v>
-      </c>
-      <c r="G1" t="s">
-        <v>305</v>
-      </c>
-      <c r="H1" t="s">
-        <v>306</v>
-      </c>
-      <c r="I1" t="s">
-        <v>307</v>
-      </c>
-      <c r="J1" t="s">
-        <v>308</v>
-      </c>
-      <c r="K1" t="s">
-        <v>309</v>
-      </c>
-      <c r="L1" t="s">
-        <v>310</v>
-      </c>
-      <c r="M1" t="s">
-        <v>311</v>
-      </c>
-      <c r="N1" t="s">
-        <v>312</v>
-      </c>
-      <c r="O1" t="s">
-        <v>313</v>
-      </c>
-      <c r="P1" t="s">
-        <v>314</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>315</v>
-      </c>
-      <c r="R1" t="s">
-        <v>328</v>
-      </c>
-      <c r="S1" t="s">
-        <v>329</v>
-      </c>
-      <c r="T1" t="s">
-        <v>330</v>
-      </c>
-      <c r="U1" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21">
-      <c r="A2" t="s">
-        <v>299</v>
-      </c>
-      <c r="B2" t="s">
-        <v>300</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>325</v>
-      </c>
-      <c r="D2" t="s">
-        <v>301</v>
-      </c>
-      <c r="F2" t="s">
-        <v>324</v>
-      </c>
-      <c r="G2" t="s">
-        <v>326</v>
-      </c>
-      <c r="H2" t="s">
-        <v>135</v>
-      </c>
-      <c r="I2" t="s">
-        <v>103</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>322</v>
-      </c>
-      <c r="K2" t="s">
-        <v>101</v>
-      </c>
-      <c r="L2" s="6" t="s">
-        <v>321</v>
-      </c>
-      <c r="M2" s="6" t="s">
-        <v>320</v>
-      </c>
-      <c r="N2" t="s">
-        <v>319</v>
-      </c>
-      <c r="O2" t="s">
-        <v>318</v>
-      </c>
-      <c r="P2" t="s">
-        <v>317</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>327</v>
-      </c>
-      <c r="R2" s="6" t="s">
-        <v>331</v>
-      </c>
-      <c r="S2" s="6" t="s">
-        <v>332</v>
-      </c>
-      <c r="T2" s="6" t="s">
-        <v>331</v>
-      </c>
-      <c r="U2" s="6" t="s">
-        <v>333</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1194F774-EACE-44AC-9C8A-A1CC70FE36E1}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="16.453125" customWidth="1"/>
-    <col min="2" max="3" width="25.54296875" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="19.26953125" customWidth="1"/>
-    <col min="6" max="6" width="14.81640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C1" t="s">
-        <v>334</v>
-      </c>
-      <c r="D1" t="s">
-        <v>136</v>
-      </c>
-      <c r="E1" t="s">
-        <v>335</v>
-      </c>
-      <c r="F1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="18.75" customHeight="1">
-      <c r="A2" t="s">
-        <v>336</v>
-      </c>
-      <c r="B2" t="s">
-        <v>337</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>338</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>339</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>340</v>
-      </c>
-      <c r="F2" t="s">
-        <v>341</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B43B544E-637D-4FD8-A2B1-2145904BBFF0}">
   <dimension ref="A1:V2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -4786,429 +5749,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01C7CE86-1D30-42A6-BFFE-DD7CB531D10C}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="16.453125" customWidth="1"/>
-    <col min="2" max="3" width="25.54296875" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="19.26953125" customWidth="1"/>
-    <col min="6" max="6" width="14.81640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C1" t="s">
-        <v>334</v>
-      </c>
-      <c r="D1" t="s">
-        <v>136</v>
-      </c>
-      <c r="E1" t="s">
-        <v>335</v>
-      </c>
-      <c r="F1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="18.75" customHeight="1">
-      <c r="A2" t="s">
-        <v>336</v>
-      </c>
-      <c r="B2" t="s">
-        <v>337</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>338</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>339</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>342</v>
-      </c>
-      <c r="F2" t="s">
-        <v>341</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06A0A6C0-CF2F-48B8-BAC5-F3E5690001A5}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="16.453125" customWidth="1"/>
-    <col min="2" max="2" width="25.54296875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
-        <v>336</v>
-      </c>
-      <c r="B2" t="s">
-        <v>337</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{120AD279-3012-4840-AF87-588B2BE3B2AA}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.81640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C1" t="s">
-        <v>130</v>
-      </c>
-      <c r="D1" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>345</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>346</v>
-      </c>
-      <c r="C2" t="s">
-        <v>347</v>
-      </c>
-      <c r="D2" t="s">
-        <v>348</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C038ED2-3C9D-4D5B-A9F6-773661E9B6A6}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C1" t="s">
-        <v>130</v>
-      </c>
-      <c r="D1" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>345</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>346</v>
-      </c>
-      <c r="C2" t="s">
-        <v>347</v>
-      </c>
-      <c r="D2" t="s">
-        <v>348</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{796CA3FD-2DF2-4849-A599-7F2B1477C186}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.81640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>345</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>346</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>349</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C6C2239-2180-4B9C-B8A1-E16F3FCE77A5}">
-  <dimension ref="A1:O2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="15.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="14.26953125" customWidth="1"/>
-    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.26953125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:15">
-      <c r="A1" t="s">
-        <v>350</v>
-      </c>
-      <c r="B1" t="s">
-        <v>351</v>
-      </c>
-      <c r="C1" t="s">
-        <v>352</v>
-      </c>
-      <c r="D1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E1" t="s">
-        <v>354</v>
-      </c>
-      <c r="F1" t="s">
-        <v>355</v>
-      </c>
-      <c r="G1" t="s">
-        <v>356</v>
-      </c>
-      <c r="H1" t="s">
-        <v>357</v>
-      </c>
-      <c r="I1" t="s">
-        <v>358</v>
-      </c>
-      <c r="J1" t="s">
-        <v>359</v>
-      </c>
-      <c r="K1" t="s">
-        <v>360</v>
-      </c>
-      <c r="L1" t="s">
-        <v>361</v>
-      </c>
-      <c r="M1" t="s">
-        <v>362</v>
-      </c>
-      <c r="N1" t="s">
-        <v>363</v>
-      </c>
-      <c r="O1" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15">
-      <c r="A2" t="s">
-        <v>365</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>366</v>
-      </c>
-      <c r="C2" s="14" t="s">
-        <v>367</v>
-      </c>
-      <c r="D2" s="14" t="s">
-        <v>368</v>
-      </c>
-      <c r="E2" s="14" t="s">
-        <v>369</v>
-      </c>
-      <c r="F2" t="s">
-        <v>370</v>
-      </c>
-      <c r="G2" t="s">
-        <v>383</v>
-      </c>
-      <c r="H2" t="s">
-        <v>101</v>
-      </c>
-      <c r="I2" t="s">
-        <v>371</v>
-      </c>
-      <c r="J2" t="s">
-        <v>372</v>
-      </c>
-      <c r="K2" t="s">
-        <v>373</v>
-      </c>
-      <c r="L2" t="s">
-        <v>374</v>
-      </c>
-      <c r="M2" s="6" t="s">
-        <v>333</v>
-      </c>
-      <c r="N2" s="6" t="s">
-        <v>375</v>
-      </c>
-      <c r="O2" t="s">
-        <v>376</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B730A7AF-1268-4970-A808-63C4CFDE9D42}">
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.26953125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>377</v>
-      </c>
-      <c r="B1" t="s">
-        <v>378</v>
-      </c>
-      <c r="C1" t="s">
-        <v>355</v>
-      </c>
-      <c r="D1" t="s">
-        <v>356</v>
-      </c>
-      <c r="E1" t="s">
-        <v>357</v>
-      </c>
-      <c r="F1" t="s">
-        <v>358</v>
-      </c>
-      <c r="G1" t="s">
-        <v>379</v>
-      </c>
-      <c r="H1" t="s">
-        <v>315</v>
-      </c>
-      <c r="I1" t="s">
-        <v>362</v>
-      </c>
-      <c r="J1" t="s">
-        <v>363</v>
-      </c>
-      <c r="K1" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11">
-      <c r="A2" s="10" t="s">
-        <v>380</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>381</v>
-      </c>
-      <c r="C2" t="s">
-        <v>370</v>
-      </c>
-      <c r="D2" t="s">
-        <v>383</v>
-      </c>
-      <c r="E2" t="s">
-        <v>101</v>
-      </c>
-      <c r="F2" t="s">
-        <v>371</v>
-      </c>
-      <c r="G2" t="s">
-        <v>373</v>
-      </c>
-      <c r="H2" t="s">
-        <v>382</v>
-      </c>
-      <c r="I2" s="6" t="s">
-        <v>333</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>375</v>
-      </c>
-      <c r="K2" t="s">
-        <v>376</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3765FB4-F532-4FCF-A614-4266393F4C44}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -5245,156 +5786,27 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3310FF1D-4559-4E35-BB7B-0285AF82C887}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-  </cols>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82EC7FC3-A185-46F7-A2D4-55C9E247ADD9}">
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="2" width="23.81640625" customWidth="1"/>
-    <col min="3" max="3" width="17.453125" customWidth="1"/>
-    <col min="4" max="4" width="22.26953125" customWidth="1"/>
-    <col min="5" max="5" width="17.453125" customWidth="1"/>
-    <col min="6" max="6" width="15.1796875" customWidth="1"/>
-    <col min="7" max="7" width="17.54296875" customWidth="1"/>
-    <col min="8" max="8" width="16.54296875" customWidth="1"/>
-    <col min="9" max="9" width="26.81640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9">
-      <c r="A1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" t="s">
-        <v>226</v>
-      </c>
-      <c r="C1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D1" t="s">
-        <v>128</v>
-      </c>
-      <c r="E1" t="s">
-        <v>119</v>
-      </c>
-      <c r="F1" t="s">
-        <v>136</v>
-      </c>
-      <c r="G1" t="s">
-        <v>121</v>
-      </c>
-      <c r="H1" t="s">
-        <v>130</v>
-      </c>
-      <c r="I1" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="18.75" customHeight="1">
-      <c r="A2" t="s">
-        <v>208</v>
-      </c>
-      <c r="B2" t="s">
-        <v>225</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="D2" t="s">
-        <v>129</v>
-      </c>
-      <c r="E2" t="s">
-        <v>120</v>
-      </c>
-      <c r="F2" s="8">
-        <v>45407</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="H2" t="s">
-        <v>131</v>
-      </c>
-      <c r="I2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{538BA7B8-E3A5-4977-A6D8-AD18062987D5}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.453125" customWidth="1"/>
-    <col min="3" max="3" width="17.453125" customWidth="1"/>
-    <col min="4" max="4" width="14.453125" customWidth="1"/>
-    <col min="5" max="5" width="16.453125" customWidth="1"/>
-    <col min="6" max="6" width="15.26953125" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C1" t="s">
-        <v>128</v>
-      </c>
-      <c r="D1" t="s">
-        <v>119</v>
-      </c>
-      <c r="E1" t="s">
-        <v>123</v>
-      </c>
-      <c r="F1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="18.75" customHeight="1">
-      <c r="A2" t="s">
-        <v>208</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="C2" t="s">
-        <v>129</v>
-      </c>
-      <c r="D2" t="s">
-        <v>135</v>
-      </c>
-      <c r="E2" s="8">
-        <v>45407</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>124</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="563c2453-77f6-4899-a3ec-7eb6553b4f66">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="c9416fa7-6169-4354-a691-3cfdebf72cd6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100957D2DE5FA4F58469907EC3226CC7D98" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="090753d51dfd09a1119d54c5de179dfc">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="563c2453-77f6-4899-a3ec-7eb6553b4f66" xmlns:ns3="c9416fa7-6169-4354-a691-3cfdebf72cd6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9c8570d9b0f0a7b9a0c34f8b658bbfee" ns2:_="" ns3:_="">
     <xsd:import namespace="563c2453-77f6-4899-a3ec-7eb6553b4f66"/>
@@ -5649,27 +6061,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="563c2453-77f6-4899-a3ec-7eb6553b4f66">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="c9416fa7-6169-4354-a691-3cfdebf72cd6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE0B556D-2173-4F7C-9F53-AE9A9D15CB9C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="563c2453-77f6-4899-a3ec-7eb6553b4f66"/>
+    <ds:schemaRef ds:uri="c9416fa7-6169-4354-a691-3cfdebf72cd6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{101DBEFA-2EFF-47B2-92EB-3E72B43EE2A6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1EC2FBF-A56D-40AC-8C09-CB1DCD191DD4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5686,23 +6097,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE0B556D-2173-4F7C-9F53-AE9A9D15CB9C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="563c2453-77f6-4899-a3ec-7eb6553b4f66"/>
-    <ds:schemaRef ds:uri="c9416fa7-6169-4354-a691-3cfdebf72cd6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{101DBEFA-2EFF-47B2-92EB-3E72B43EE2A6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Change in medication Excel
</commit_message>
<xml_diff>
--- a/ExcelFiles/PatientSummary.xlsx
+++ b/ExcelFiles/PatientSummary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Cellma4ClinicalAuto2\Cellma4ClinicalAuto2\ExcelFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Riomed\Cellma4ClinicalAuto2\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A94AE17-6DCC-4CA5-9AE7-B286177A44A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69538DD9-19D1-43DF-B65C-6291795EB876}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="55" activeTab="60" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loginDetails" sheetId="2" r:id="rId1"/>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="948" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="441">
   <si>
     <t>username</t>
   </si>
@@ -378,9 +378,6 @@
   </si>
   <si>
     <t>Drowsiness</t>
-  </si>
-  <si>
-    <t>Aspirin 25mg capsules</t>
   </si>
   <si>
     <t>pacr_status</t>
@@ -1799,18 +1796,18 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>375</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>376</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>377</v>
       </c>
     </row>
   </sheetData>
@@ -1836,15 +1833,15 @@
         <v>67</v>
       </c>
       <c r="B1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -1870,39 +1867,39 @@
         <v>67</v>
       </c>
       <c r="B1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C1" t="s">
         <v>68</v>
       </c>
       <c r="D1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -1930,30 +1927,30 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -1978,18 +1975,18 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -2018,54 +2015,54 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E1" t="s">
+        <v>146</v>
+      </c>
+      <c r="F1" t="s">
         <v>147</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>148</v>
       </c>
-      <c r="G1" t="s">
-        <v>149</v>
-      </c>
       <c r="H1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B2" t="s">
         <v>150</v>
-      </c>
-      <c r="B2" t="s">
-        <v>151</v>
       </c>
       <c r="C2" s="9">
         <v>45420</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="H2" t="s">
         <v>152</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>153</v>
-      </c>
-      <c r="I2" t="s">
-        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -2097,54 +2094,54 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E1" t="s">
+        <v>146</v>
+      </c>
+      <c r="F1" t="s">
         <v>147</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>148</v>
       </c>
-      <c r="G1" t="s">
-        <v>149</v>
-      </c>
       <c r="H1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B2" t="s">
         <v>150</v>
       </c>
-      <c r="B2" t="s">
-        <v>151</v>
-      </c>
       <c r="C2" s="10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>82</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="H2" t="s">
         <v>156</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>157</v>
-      </c>
-      <c r="I2" t="s">
-        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -2166,15 +2163,15 @@
         <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -2205,81 +2202,81 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1" t="s">
         <v>95</v>
       </c>
-      <c r="D1" t="s">
-        <v>96</v>
-      </c>
       <c r="E1" t="s">
+        <v>138</v>
+      </c>
+      <c r="F1" t="s">
         <v>139</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>140</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>141</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
+        <v>143</v>
+      </c>
+      <c r="J1" t="s">
         <v>142</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>144</v>
       </c>
-      <c r="J1" t="s">
-        <v>143</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>145</v>
       </c>
-      <c r="L1" t="s">
-        <v>146</v>
-      </c>
       <c r="M1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="N1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B2" t="s">
         <v>135</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>136</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>137</v>
       </c>
-      <c r="D2" t="s">
-        <v>138</v>
-      </c>
       <c r="E2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F2" t="s">
+        <v>159</v>
+      </c>
+      <c r="G2" t="s">
         <v>160</v>
       </c>
-      <c r="G2" t="s">
-        <v>161</v>
-      </c>
       <c r="I2" s="10" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="K2" s="10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="M2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="N2" s="9" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -2311,69 +2308,69 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1" t="s">
         <v>95</v>
       </c>
-      <c r="D1" t="s">
-        <v>96</v>
-      </c>
       <c r="E1" t="s">
+        <v>138</v>
+      </c>
+      <c r="F1" t="s">
         <v>139</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>140</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>141</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
+        <v>143</v>
+      </c>
+      <c r="J1" t="s">
         <v>142</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>144</v>
       </c>
-      <c r="J1" t="s">
-        <v>143</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>145</v>
-      </c>
-      <c r="L1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B2" t="s">
         <v>135</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>136</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>137</v>
       </c>
-      <c r="D2" t="s">
-        <v>138</v>
-      </c>
       <c r="E2" t="s">
+        <v>163</v>
+      </c>
+      <c r="F2" t="s">
         <v>164</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>165</v>
       </c>
-      <c r="G2" t="s">
-        <v>166</v>
-      </c>
       <c r="I2" s="10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K2" s="10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -2395,15 +2392,15 @@
         <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -2570,22 +2567,22 @@
     </row>
     <row r="2" spans="1:48" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F2" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>433</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>434</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>50</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>51</v>
@@ -2683,36 +2680,36 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
+        <v>172</v>
+      </c>
+      <c r="D1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E1" t="s">
         <v>173</v>
       </c>
-      <c r="D1" t="s">
-        <v>134</v>
-      </c>
-      <c r="E1" t="s">
-        <v>174</v>
-      </c>
       <c r="F1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D2" s="8">
         <v>45453</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -2741,36 +2738,36 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
+        <v>172</v>
+      </c>
+      <c r="D1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E1" t="s">
         <v>173</v>
       </c>
-      <c r="D1" t="s">
-        <v>134</v>
-      </c>
-      <c r="E1" t="s">
-        <v>174</v>
-      </c>
       <c r="F1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D2" s="8">
         <v>45453</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -2796,18 +2793,18 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -2839,49 +2836,49 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D2" s="7" t="str">
         <f ca="1">TEXT(TODAY(), "DD/MM/YYYY")</f>
-        <v>28/05/2025</v>
+        <v>04/06/2025</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G2" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="H2" s="10" t="s">
         <v>285</v>
-      </c>
-      <c r="H2" s="10" t="s">
-        <v>286</v>
       </c>
       <c r="I2" s="8"/>
     </row>
@@ -2913,49 +2910,49 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D2" s="7" t="str">
         <f ca="1">TEXT(TODAY(), "DD/MM/YYYY")</f>
-        <v>28/05/2025</v>
+        <v>04/06/2025</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G2" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="H2" s="7" t="s">
         <v>286</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>287</v>
       </c>
     </row>
   </sheetData>
@@ -2981,18 +2978,18 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -3027,84 +3024,84 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D1" t="s">
+        <v>208</v>
+      </c>
+      <c r="E1" t="s">
         <v>209</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>210</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
+        <v>214</v>
+      </c>
+      <c r="H1" t="s">
         <v>211</v>
       </c>
-      <c r="G1" t="s">
-        <v>215</v>
-      </c>
-      <c r="H1" t="s">
-        <v>212</v>
-      </c>
       <c r="I1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="J1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L1" t="s">
+        <v>205</v>
+      </c>
+      <c r="M1" t="s">
         <v>206</v>
       </c>
-      <c r="M1" t="s">
-        <v>207</v>
-      </c>
       <c r="N1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B2" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="J2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="K2" s="8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="M2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="N2" s="9" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -3135,73 +3132,73 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
+        <v>208</v>
+      </c>
+      <c r="D1" t="s">
         <v>209</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>210</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>214</v>
+      </c>
+      <c r="G1" t="s">
         <v>211</v>
       </c>
-      <c r="F1" t="s">
-        <v>215</v>
-      </c>
-      <c r="G1" t="s">
-        <v>212</v>
-      </c>
       <c r="H1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="K1" t="s">
+        <v>205</v>
+      </c>
+      <c r="L1" t="s">
         <v>206</v>
-      </c>
-      <c r="L1" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B2" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C2" s="7">
         <f ca="1">TODAY()</f>
-        <v>45805</v>
+        <v>45812</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="I2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="K2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
   </sheetData>
@@ -3227,18 +3224,18 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B2" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -3262,57 +3259,57 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D1" t="s">
+        <v>224</v>
+      </c>
+      <c r="E1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F1" t="s">
         <v>225</v>
       </c>
-      <c r="E1" t="s">
-        <v>128</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
+        <v>129</v>
+      </c>
+      <c r="H1" s="11" t="s">
         <v>226</v>
       </c>
-      <c r="G1" t="s">
-        <v>130</v>
-      </c>
-      <c r="H1" s="11" t="s">
+      <c r="I1" s="11" t="s">
         <v>227</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="J1" s="11" t="s">
         <v>228</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="K1" s="11" t="s">
         <v>229</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="L1" t="s">
         <v>230</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>231</v>
-      </c>
-      <c r="M1" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>232</v>
+      </c>
+      <c r="B2" t="s">
         <v>233</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="C2" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" t="s">
         <v>235</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>236</v>
-      </c>
-      <c r="F2" t="s">
-        <v>237</v>
       </c>
       <c r="G2">
         <v>57749615244</v>
@@ -3321,19 +3318,19 @@
         <v>82</v>
       </c>
       <c r="I2" s="12" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="J2" s="12" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="K2" s="12" t="s">
+        <v>237</v>
+      </c>
+      <c r="L2" t="s">
         <v>238</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>239</v>
-      </c>
-      <c r="M2" t="s">
-        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -3378,78 +3375,78 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D1" t="s">
+        <v>224</v>
+      </c>
+      <c r="E1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F1" t="s">
+        <v>129</v>
+      </c>
+      <c r="G1" s="11" t="s">
         <v>225</v>
       </c>
-      <c r="E1" t="s">
-        <v>128</v>
-      </c>
-      <c r="F1" t="s">
-        <v>130</v>
-      </c>
-      <c r="G1" s="11" t="s">
+      <c r="H1" s="11" t="s">
         <v>226</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="I1" s="11" t="s">
         <v>227</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="J1" s="11" t="s">
         <v>228</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="K1" s="11" t="s">
         <v>229</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="L1" t="s">
         <v>230</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>231</v>
-      </c>
-      <c r="M1" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>232</v>
+      </c>
+      <c r="B2" t="s">
         <v>233</v>
       </c>
-      <c r="B2" t="s">
-        <v>234</v>
-      </c>
       <c r="C2" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F2">
         <v>57749615244</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="H2" s="12" t="s">
         <v>82</v>
       </c>
       <c r="I2" s="12" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="J2" s="12" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="K2" s="12" t="s">
+        <v>237</v>
+      </c>
+      <c r="L2" t="s">
         <v>238</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>239</v>
-      </c>
-      <c r="M2" t="s">
-        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -3471,15 +3468,15 @@
         <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -3513,66 +3510,66 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D1" t="s">
+        <v>241</v>
+      </c>
+      <c r="E1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F1" t="s">
         <v>242</v>
       </c>
-      <c r="E1" t="s">
-        <v>128</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
+        <v>129</v>
+      </c>
+      <c r="H1" s="11" t="s">
         <v>243</v>
       </c>
-      <c r="G1" t="s">
-        <v>130</v>
-      </c>
-      <c r="H1" s="11" t="s">
+      <c r="I1" s="11" t="s">
         <v>244</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="J1" s="11" t="s">
         <v>245</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="K1" s="11" t="s">
         <v>246</v>
-      </c>
-      <c r="K1" s="11" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>247</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>439</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>440</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" t="s">
         <v>249</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" s="12" t="s">
         <v>250</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="G2" t="s">
         <v>251</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" s="12" t="s">
         <v>252</v>
       </c>
-      <c r="H2" s="12" t="s">
+      <c r="I2" s="12" t="s">
         <v>253</v>
       </c>
-      <c r="I2" s="12" t="s">
-        <v>254</v>
-      </c>
       <c r="J2" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="K2" s="12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -3606,66 +3603,66 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D1" t="s">
+        <v>241</v>
+      </c>
+      <c r="E1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F1" t="s">
         <v>242</v>
       </c>
-      <c r="E1" t="s">
-        <v>128</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
+        <v>129</v>
+      </c>
+      <c r="H1" s="11" t="s">
         <v>243</v>
       </c>
-      <c r="G1" t="s">
-        <v>130</v>
-      </c>
-      <c r="H1" s="11" t="s">
+      <c r="I1" s="11" t="s">
         <v>244</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="J1" s="11" t="s">
         <v>245</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="K1" s="11" t="s">
         <v>246</v>
-      </c>
-      <c r="K1" s="11" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="E2" t="s">
+        <v>249</v>
+      </c>
+      <c r="F2" s="12" t="s">
         <v>255</v>
       </c>
-      <c r="E2" t="s">
-        <v>250</v>
-      </c>
-      <c r="F2" s="12" t="s">
+      <c r="G2" t="s">
+        <v>251</v>
+      </c>
+      <c r="H2" s="12" t="s">
         <v>256</v>
       </c>
-      <c r="G2" t="s">
-        <v>252</v>
-      </c>
-      <c r="H2" s="12" t="s">
+      <c r="I2" s="12" t="s">
         <v>257</v>
       </c>
-      <c r="I2" s="12" t="s">
-        <v>258</v>
-      </c>
       <c r="J2" s="12" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K2" s="12" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -3687,15 +3684,15 @@
         <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
   </sheetData>
@@ -3724,33 +3721,33 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D1" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>260</v>
+      </c>
+      <c r="B2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>261</v>
       </c>
-      <c r="B2" t="s">
-        <v>261</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" t="s">
         <v>262</v>
-      </c>
-      <c r="E2" t="s">
-        <v>263</v>
       </c>
       <c r="F2">
         <v>5774961523</v>
@@ -3780,24 +3777,24 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
   </sheetData>
@@ -3819,15 +3816,15 @@
         <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -3854,24 +3851,24 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B2" t="s">
+        <v>264</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" t="s">
         <v>266</v>
-      </c>
-      <c r="D2" t="s">
-        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -3898,24 +3895,24 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D2" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -3981,7 +3978,7 @@
         <v>74</v>
       </c>
       <c r="H1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I1" t="s">
         <v>75</v>
@@ -3990,10 +3987,10 @@
         <v>76</v>
       </c>
       <c r="K1" t="s">
+        <v>94</v>
+      </c>
+      <c r="L1" t="s">
         <v>95</v>
-      </c>
-      <c r="L1" t="s">
-        <v>96</v>
       </c>
       <c r="M1" t="s">
         <v>79</v>
@@ -4002,10 +3999,10 @@
         <v>80</v>
       </c>
       <c r="O1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="P1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="Q1" t="s">
         <v>84</v>
@@ -4017,51 +4014,51 @@
         <v>92</v>
       </c>
       <c r="T1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="U1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="V1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="W1" t="s">
+        <v>106</v>
+      </c>
+      <c r="X1" t="s">
+        <v>104</v>
+      </c>
+      <c r="Y1" t="s">
         <v>107</v>
       </c>
-      <c r="X1" t="s">
-        <v>105</v>
-      </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>108</v>
       </c>
-      <c r="Z1" t="s">
-        <v>109</v>
-      </c>
       <c r="AA1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AB1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AC1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AD1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AE1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AF1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B2" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>82</v>
@@ -4079,25 +4076,25 @@
         <v>82</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I2" s="7" t="s">
+        <v>435</v>
+      </c>
+      <c r="J2" s="7" t="s">
         <v>436</v>
       </c>
-      <c r="J2" s="7" t="s">
-        <v>437</v>
-      </c>
       <c r="K2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="N2" t="s">
         <v>83</v>
       </c>
       <c r="O2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="P2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="Q2" t="s">
         <v>85</v>
@@ -4109,43 +4106,43 @@
         <v>93</v>
       </c>
       <c r="T2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="U2" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="V2" s="6" t="s">
         <v>82</v>
       </c>
       <c r="W2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="X2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="Y2" s="6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="Z2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="AA2" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="AB2">
         <v>5</v>
       </c>
       <c r="AC2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="AD2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AE2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AF2" s="9" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -4171,18 +4168,18 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -4209,24 +4206,24 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
   </sheetData>
@@ -4253,24 +4250,24 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>274</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>332</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>276</v>
-      </c>
       <c r="D2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
   </sheetData>
@@ -4296,18 +4293,18 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
   </sheetData>
@@ -4333,24 +4330,24 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
   </sheetData>
@@ -4376,24 +4373,24 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>279</v>
+      </c>
+      <c r="B2" t="s">
+        <v>373</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="B2" t="s">
-        <v>374</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>281</v>
-      </c>
       <c r="D2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
   </sheetData>
@@ -4419,18 +4416,18 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
   </sheetData>
@@ -4460,99 +4457,99 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
+        <v>290</v>
+      </c>
+      <c r="D1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E1" t="s">
         <v>291</v>
       </c>
-      <c r="D1" t="s">
-        <v>128</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>292</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>293</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>294</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>295</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>296</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>297</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>298</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>299</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>300</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>301</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>302</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>303</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>287</v>
+      </c>
+      <c r="B2" t="s">
         <v>288</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="D2" t="s">
         <v>289</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>208</v>
-      </c>
-      <c r="D2" t="s">
-        <v>290</v>
-      </c>
       <c r="F2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="G2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="K2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="N2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="O2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="P2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="Q2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
   </sheetData>
@@ -4583,123 +4580,123 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
+        <v>290</v>
+      </c>
+      <c r="D1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E1" t="s">
         <v>291</v>
       </c>
-      <c r="D1" t="s">
-        <v>128</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>292</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>293</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>294</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>295</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>296</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>297</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>298</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>299</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>300</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>301</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>302</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>303</v>
       </c>
-      <c r="Q1" t="s">
-        <v>304</v>
-      </c>
       <c r="R1" t="s">
+        <v>316</v>
+      </c>
+      <c r="S1" t="s">
         <v>317</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>318</v>
       </c>
-      <c r="T1" t="s">
-        <v>319</v>
-      </c>
       <c r="U1" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>287</v>
+      </c>
+      <c r="B2" t="s">
         <v>288</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="D2" t="s">
         <v>289</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="F2" t="s">
+        <v>312</v>
+      </c>
+      <c r="G2" t="s">
         <v>314</v>
       </c>
-      <c r="D2" t="s">
-        <v>290</v>
-      </c>
-      <c r="F2" t="s">
-        <v>313</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
+        <v>132</v>
+      </c>
+      <c r="I2" t="s">
+        <v>100</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="K2" t="s">
+        <v>98</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="N2" t="s">
+        <v>307</v>
+      </c>
+      <c r="O2" t="s">
+        <v>306</v>
+      </c>
+      <c r="P2" t="s">
+        <v>305</v>
+      </c>
+      <c r="Q2" t="s">
         <v>315</v>
       </c>
-      <c r="H2" t="s">
-        <v>133</v>
-      </c>
-      <c r="I2" t="s">
-        <v>101</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>311</v>
-      </c>
-      <c r="K2" t="s">
-        <v>99</v>
-      </c>
-      <c r="L2" s="6" t="s">
-        <v>310</v>
-      </c>
-      <c r="M2" s="6" t="s">
-        <v>309</v>
-      </c>
-      <c r="N2" t="s">
-        <v>308</v>
-      </c>
-      <c r="O2" t="s">
-        <v>307</v>
-      </c>
-      <c r="P2" t="s">
-        <v>306</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>316</v>
-      </c>
       <c r="R2" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="S2" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="S2" s="6" t="s">
+      <c r="T2" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="U2" s="6" t="s">
         <v>321</v>
-      </c>
-      <c r="T2" s="6" t="s">
-        <v>320</v>
-      </c>
-      <c r="U2" s="6" t="s">
-        <v>322</v>
       </c>
     </row>
   </sheetData>
@@ -4727,36 +4724,36 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
+        <v>322</v>
+      </c>
+      <c r="D1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E1" t="s">
         <v>323</v>
       </c>
-      <c r="D1" t="s">
-        <v>134</v>
-      </c>
-      <c r="E1" t="s">
-        <v>324</v>
-      </c>
       <c r="F1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>324</v>
+      </c>
+      <c r="B2" t="s">
         <v>325</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="7" t="s">
         <v>326</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="7" t="s">
         <v>327</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="E2" s="3" t="s">
         <v>328</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" t="s">
         <v>329</v>
-      </c>
-      <c r="F2" t="s">
-        <v>330</v>
       </c>
     </row>
   </sheetData>
@@ -4808,7 +4805,7 @@
         <v>81</v>
       </c>
       <c r="G1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H1" t="s">
         <v>74</v>
@@ -4835,36 +4832,37 @@
         <v>84</v>
       </c>
       <c r="P1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q1" t="s">
         <v>92</v>
       </c>
       <c r="R1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="S1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="T1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="U1" t="s">
         <v>84</v>
       </c>
       <c r="V1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>224</v>
-      </c>
-      <c r="B2" t="s">
-        <v>439</v>
+        <v>223</v>
+      </c>
+      <c r="B2" t="str">
+        <f>AddMedication!B2</f>
+        <v>Paracetamol 500mg / Ibuprofen 200mg tablets</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D2" t="s">
         <v>86</v>
@@ -4876,16 +4874,16 @@
         <v>73</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I2" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="J2" s="7" t="s">
         <v>184</v>
-      </c>
-      <c r="J2" s="7" t="s">
-        <v>185</v>
       </c>
       <c r="K2" t="s">
         <v>89</v>
@@ -4897,25 +4895,25 @@
         <v>88</v>
       </c>
       <c r="P2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="Q2" t="s">
         <v>93</v>
       </c>
       <c r="R2" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="S2" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="T2" t="s">
+        <v>186</v>
+      </c>
+      <c r="U2" t="s">
         <v>188</v>
       </c>
-      <c r="T2" t="s">
-        <v>187</v>
-      </c>
-      <c r="U2" t="s">
-        <v>189</v>
-      </c>
       <c r="V2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -4943,36 +4941,36 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
+        <v>322</v>
+      </c>
+      <c r="D1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E1" t="s">
         <v>323</v>
       </c>
-      <c r="D1" t="s">
-        <v>134</v>
-      </c>
-      <c r="E1" t="s">
-        <v>324</v>
-      </c>
       <c r="F1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>324</v>
+      </c>
+      <c r="B2" t="s">
         <v>325</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="7" t="s">
         <v>326</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="7" t="s">
         <v>327</v>
       </c>
-      <c r="D2" s="7" t="s">
-        <v>328</v>
-      </c>
       <c r="E2" s="3" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F2" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
   </sheetData>
@@ -4999,10 +4997,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>324</v>
+      </c>
+      <c r="B2" t="s">
         <v>325</v>
-      </c>
-      <c r="B2" t="s">
-        <v>326</v>
       </c>
     </row>
   </sheetData>
@@ -5029,24 +5027,24 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D1" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>333</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C2" t="s">
         <v>335</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>336</v>
-      </c>
-      <c r="D2" t="s">
-        <v>337</v>
       </c>
     </row>
   </sheetData>
@@ -5074,24 +5072,24 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D1" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>333</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C2" t="s">
         <v>335</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>336</v>
-      </c>
-      <c r="D2" t="s">
-        <v>337</v>
       </c>
     </row>
   </sheetData>
@@ -5117,18 +5115,18 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>333</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>335</v>
-      </c>
       <c r="C2" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
   </sheetData>
@@ -5157,96 +5155,96 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>338</v>
+      </c>
+      <c r="B1" t="s">
         <v>339</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>340</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>341</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>342</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>343</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>344</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>345</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>346</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>347</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>348</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>349</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>350</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>351</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>352</v>
-      </c>
-      <c r="O1" t="s">
-        <v>353</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>353</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>354</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="C2" s="13" t="s">
         <v>355</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="D2" s="13" t="s">
         <v>356</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="E2" s="13" t="s">
         <v>357</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="F2" t="s">
         <v>358</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
+        <v>371</v>
+      </c>
+      <c r="H2" t="s">
+        <v>98</v>
+      </c>
+      <c r="I2" t="s">
         <v>359</v>
       </c>
-      <c r="G2" t="s">
-        <v>372</v>
-      </c>
-      <c r="H2" t="s">
-        <v>99</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>360</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>361</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>362</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="N2" s="6" t="s">
         <v>363</v>
       </c>
-      <c r="M2" s="6" t="s">
-        <v>322</v>
-      </c>
-      <c r="N2" s="6" t="s">
+      <c r="O2" t="s">
         <v>364</v>
-      </c>
-      <c r="O2" t="s">
-        <v>365</v>
       </c>
     </row>
   </sheetData>
@@ -5272,72 +5270,72 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>365</v>
+      </c>
+      <c r="B1" t="s">
         <v>366</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>343</v>
+      </c>
+      <c r="D1" t="s">
+        <v>344</v>
+      </c>
+      <c r="E1" t="s">
+        <v>345</v>
+      </c>
+      <c r="F1" t="s">
+        <v>346</v>
+      </c>
+      <c r="G1" t="s">
         <v>367</v>
       </c>
-      <c r="C1" t="s">
-        <v>344</v>
-      </c>
-      <c r="D1" t="s">
-        <v>345</v>
-      </c>
-      <c r="E1" t="s">
-        <v>346</v>
-      </c>
-      <c r="F1" t="s">
-        <v>347</v>
-      </c>
-      <c r="G1" t="s">
-        <v>368</v>
-      </c>
       <c r="H1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="I1" t="s">
+        <v>350</v>
+      </c>
+      <c r="J1" t="s">
         <v>351</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>352</v>
-      </c>
-      <c r="K1" t="s">
-        <v>353</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
+        <v>368</v>
+      </c>
+      <c r="B2" s="13" t="s">
         <v>369</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="C2" t="s">
+        <v>358</v>
+      </c>
+      <c r="D2" t="s">
+        <v>371</v>
+      </c>
+      <c r="E2" t="s">
+        <v>98</v>
+      </c>
+      <c r="F2" t="s">
+        <v>359</v>
+      </c>
+      <c r="G2" t="s">
+        <v>361</v>
+      </c>
+      <c r="H2" t="s">
         <v>370</v>
       </c>
-      <c r="C2" t="s">
-        <v>359</v>
-      </c>
-      <c r="D2" t="s">
-        <v>372</v>
-      </c>
-      <c r="E2" t="s">
-        <v>99</v>
-      </c>
-      <c r="F2" t="s">
-        <v>360</v>
-      </c>
-      <c r="G2" t="s">
-        <v>362</v>
-      </c>
-      <c r="H2" t="s">
-        <v>371</v>
-      </c>
       <c r="I2" s="6" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="J2" s="6" t="s">
+        <v>363</v>
+      </c>
+      <c r="K2" t="s">
         <v>364</v>
-      </c>
-      <c r="K2" t="s">
-        <v>365</v>
       </c>
     </row>
   </sheetData>
@@ -5373,93 +5371,93 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
+        <v>380</v>
+      </c>
+      <c r="D1" t="s">
         <v>381</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>382</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>383</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>384</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>385</v>
       </c>
-      <c r="H1" t="s">
-        <v>386</v>
-      </c>
       <c r="I1" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="J1" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="K1" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="L1" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="M1" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="N1" t="s">
+        <v>402</v>
+      </c>
+      <c r="O1" t="s">
         <v>403</v>
-      </c>
-      <c r="O1" t="s">
-        <v>404</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>405</v>
+      </c>
+      <c r="B2" t="s">
+        <v>379</v>
+      </c>
+      <c r="C2" t="s">
+        <v>386</v>
+      </c>
+      <c r="D2" t="s">
+        <v>387</v>
+      </c>
+      <c r="E2" t="s">
+        <v>388</v>
+      </c>
+      <c r="F2" t="s">
+        <v>389</v>
+      </c>
+      <c r="G2" t="s">
+        <v>390</v>
+      </c>
+      <c r="H2" t="s">
+        <v>391</v>
+      </c>
+      <c r="I2" t="s">
+        <v>393</v>
+      </c>
+      <c r="J2" t="s">
+        <v>395</v>
+      </c>
+      <c r="K2" t="s">
+        <v>397</v>
+      </c>
+      <c r="L2" t="s">
+        <v>399</v>
+      </c>
+      <c r="M2" t="s">
+        <v>401</v>
+      </c>
+      <c r="N2" t="s">
         <v>406</v>
       </c>
-      <c r="B2" t="s">
-        <v>380</v>
-      </c>
-      <c r="C2" t="s">
-        <v>387</v>
-      </c>
-      <c r="D2" t="s">
-        <v>388</v>
-      </c>
-      <c r="E2" t="s">
-        <v>389</v>
-      </c>
-      <c r="F2" t="s">
-        <v>390</v>
-      </c>
-      <c r="G2" t="s">
-        <v>391</v>
-      </c>
-      <c r="H2" t="s">
-        <v>392</v>
-      </c>
-      <c r="I2" t="s">
-        <v>394</v>
-      </c>
-      <c r="J2" t="s">
-        <v>396</v>
-      </c>
-      <c r="K2" t="s">
-        <v>398</v>
-      </c>
-      <c r="L2" t="s">
-        <v>400</v>
-      </c>
-      <c r="M2" t="s">
-        <v>402</v>
-      </c>
-      <c r="N2" t="s">
-        <v>407</v>
-      </c>
       <c r="O2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="P2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
   </sheetData>
@@ -5495,93 +5493,93 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
+        <v>380</v>
+      </c>
+      <c r="D1" t="s">
         <v>381</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>382</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>383</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>384</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>385</v>
       </c>
-      <c r="H1" t="s">
-        <v>386</v>
-      </c>
       <c r="I1" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="J1" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="K1" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="L1" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="M1" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="N1" t="s">
+        <v>402</v>
+      </c>
+      <c r="O1" t="s">
         <v>403</v>
-      </c>
-      <c r="O1" t="s">
-        <v>404</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C2" t="s">
+        <v>386</v>
+      </c>
+      <c r="D2" t="s">
         <v>387</v>
       </c>
-      <c r="D2" t="s">
-        <v>388</v>
-      </c>
       <c r="E2" t="s">
+        <v>407</v>
+      </c>
+      <c r="F2" t="s">
+        <v>389</v>
+      </c>
+      <c r="G2" t="s">
+        <v>390</v>
+      </c>
+      <c r="H2" t="s">
         <v>408</v>
       </c>
-      <c r="F2" t="s">
-        <v>390</v>
-      </c>
-      <c r="G2" t="s">
-        <v>391</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
+        <v>393</v>
+      </c>
+      <c r="J2" t="s">
+        <v>395</v>
+      </c>
+      <c r="K2" t="s">
         <v>409</v>
       </c>
-      <c r="I2" t="s">
-        <v>394</v>
-      </c>
-      <c r="J2" t="s">
-        <v>396</v>
-      </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
+        <v>399</v>
+      </c>
+      <c r="M2" t="s">
+        <v>401</v>
+      </c>
+      <c r="N2" t="s">
         <v>410</v>
       </c>
-      <c r="L2" t="s">
-        <v>400</v>
-      </c>
-      <c r="M2" t="s">
-        <v>402</v>
-      </c>
-      <c r="N2" t="s">
-        <v>411</v>
-      </c>
       <c r="O2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="P2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
   </sheetData>
@@ -5616,18 +5614,19 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>224</v>
-      </c>
-      <c r="B2" t="s">
-        <v>94</v>
+        <v>223</v>
+      </c>
+      <c r="B2" t="str">
+        <f>EditMedication!B2</f>
+        <v>Paracetamol 500mg / Ibuprofen 200mg tablets</v>
       </c>
       <c r="C2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -5655,76 +5654,76 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>411</v>
+      </c>
+      <c r="B1" t="s">
         <v>412</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>413</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>414</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>415</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>416</v>
       </c>
-      <c r="F1" t="s">
-        <v>417</v>
-      </c>
       <c r="G1" t="s">
+        <v>419</v>
+      </c>
+      <c r="H1" t="s">
         <v>420</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>421</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>422</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>423</v>
       </c>
-      <c r="K1" t="s">
-        <v>424</v>
-      </c>
       <c r="L1" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B2" s="8" t="str">
         <f ca="1">TEXT(TODAY(), "DD/MM/YYYY")</f>
-        <v>28/05/2025</v>
+        <v>04/06/2025</v>
       </c>
       <c r="C2" t="s">
+        <v>417</v>
+      </c>
+      <c r="D2" t="s">
         <v>418</v>
       </c>
-      <c r="D2" t="s">
-        <v>419</v>
-      </c>
       <c r="E2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H2" t="s">
+        <v>424</v>
+      </c>
+      <c r="I2" t="s">
         <v>425</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>426</v>
       </c>
-      <c r="J2" t="s">
-        <v>427</v>
-      </c>
       <c r="K2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="L2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
   </sheetData>
@@ -5754,99 +5753,99 @@
         <v>68</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E1" t="s">
+        <v>291</v>
+      </c>
+      <c r="F1" t="s">
         <v>292</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>293</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>294</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>295</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>296</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>297</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>298</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>299</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>300</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>301</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>302</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>303</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>287</v>
+      </c>
+      <c r="B2" t="s">
         <v>288</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="D2" t="s">
         <v>289</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="D2" t="s">
-        <v>290</v>
-      </c>
       <c r="F2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="G2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="K2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="N2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="O2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="P2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="Q2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
   </sheetData>
@@ -5887,57 +5886,57 @@
         <v>67</v>
       </c>
       <c r="B1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C1" t="s">
         <v>68</v>
       </c>
       <c r="D1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F2" s="8">
         <v>45407</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -5967,36 +5966,36 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E2" s="8">
         <v>45407</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add form in Add medication
</commit_message>
<xml_diff>
--- a/ExcelFiles/PatientSummary.xlsx
+++ b/ExcelFiles/PatientSummary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Riomed\Cellma4ClinicalAuto2\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DDD059A-93DD-4F1E-93C1-ABA8B0A9A079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F0575D3-1E3C-4F9B-A3AF-139E934B1A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="2250" yWindow="2250" windowWidth="18000" windowHeight="9270" firstSheet="23" activeTab="25" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loginDetails" sheetId="2" r:id="rId1"/>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="947" uniqueCount="442">
   <si>
     <t>username</t>
   </si>
@@ -1419,6 +1419,9 @@
   </si>
   <si>
     <t>Knee Arthroplasty</t>
+  </si>
+  <si>
+    <t>medi_form</t>
   </si>
 </sst>
 </file>
@@ -2866,7 +2869,7 @@
       </c>
       <c r="D2" s="7" t="str">
         <f ca="1">TEXT(TODAY(), "DD/MM/YYYY")</f>
-        <v>04/06/2025</v>
+        <v>09/06/2025</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>198</v>
@@ -2940,7 +2943,7 @@
       </c>
       <c r="D2" s="7" t="str">
         <f ca="1">TEXT(TODAY(), "DD/MM/YYYY")</f>
-        <v>04/06/2025</v>
+        <v>09/06/2025</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>199</v>
@@ -3171,7 +3174,7 @@
       </c>
       <c r="C2" s="7">
         <f ca="1">TODAY()</f>
-        <v>45812</v>
+        <v>45817</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>103</v>
@@ -3922,40 +3925,40 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DD9439C-0973-45AC-88BC-21584AF7E144}">
-  <dimension ref="A1:AF2"/>
+  <dimension ref="A1:AG2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.42578125" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="8" width="13.7109375" customWidth="1"/>
-    <col min="9" max="9" width="11.85546875" customWidth="1"/>
-    <col min="10" max="10" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.42578125" customWidth="1"/>
-    <col min="12" max="12" width="12.5703125" customWidth="1"/>
-    <col min="13" max="13" width="17" customWidth="1"/>
-    <col min="14" max="16" width="15.5703125" customWidth="1"/>
-    <col min="17" max="17" width="12.85546875" customWidth="1"/>
-    <col min="18" max="18" width="16.5703125" customWidth="1"/>
-    <col min="19" max="20" width="16" customWidth="1"/>
-    <col min="21" max="21" width="13.140625" customWidth="1"/>
-    <col min="22" max="22" width="21" customWidth="1"/>
-    <col min="23" max="23" width="13.140625" customWidth="1"/>
-    <col min="24" max="24" width="17.7109375" customWidth="1"/>
-    <col min="25" max="25" width="13.85546875" customWidth="1"/>
-    <col min="26" max="26" width="12.28515625" customWidth="1"/>
-    <col min="27" max="27" width="15.140625" customWidth="1"/>
-    <col min="28" max="28" width="28.42578125" customWidth="1"/>
-    <col min="29" max="29" width="14.85546875" customWidth="1"/>
-    <col min="30" max="30" width="17.140625" customWidth="1"/>
-    <col min="31" max="31" width="27.140625" customWidth="1"/>
-    <col min="32" max="32" width="12.85546875" customWidth="1"/>
+    <col min="3" max="4" width="17.7109375" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="9" width="13.7109375" customWidth="1"/>
+    <col min="10" max="10" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.42578125" customWidth="1"/>
+    <col min="13" max="13" width="12.5703125" customWidth="1"/>
+    <col min="14" max="14" width="17" customWidth="1"/>
+    <col min="15" max="17" width="15.5703125" customWidth="1"/>
+    <col min="18" max="18" width="12.85546875" customWidth="1"/>
+    <col min="19" max="19" width="16.5703125" customWidth="1"/>
+    <col min="20" max="21" width="16" customWidth="1"/>
+    <col min="22" max="22" width="13.140625" customWidth="1"/>
+    <col min="23" max="23" width="21" customWidth="1"/>
+    <col min="24" max="24" width="13.140625" customWidth="1"/>
+    <col min="25" max="25" width="17.7109375" customWidth="1"/>
+    <col min="26" max="26" width="13.85546875" customWidth="1"/>
+    <col min="27" max="27" width="12.28515625" customWidth="1"/>
+    <col min="28" max="28" width="15.140625" customWidth="1"/>
+    <col min="29" max="29" width="28.42578125" customWidth="1"/>
+    <col min="30" max="30" width="14.85546875" customWidth="1"/>
+    <col min="31" max="31" width="17.140625" customWidth="1"/>
+    <col min="32" max="32" width="27.140625" customWidth="1"/>
+    <col min="33" max="33" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -3966,182 +3969,188 @@
         <v>69</v>
       </c>
       <c r="D1" t="s">
+        <v>441</v>
+      </c>
+      <c r="E1" t="s">
         <v>70</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>72</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>81</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>74</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>101</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>75</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>76</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>94</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>95</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>79</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>80</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>97</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>179</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>84</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>90</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>92</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>99</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>96</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>114</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>106</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>104</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>107</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>108</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>110</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>107</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AD1" t="s">
         <v>112</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AE1" t="s">
         <v>127</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AF1" t="s">
         <v>181</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AG1" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>223</v>
       </c>
       <c r="B2" t="s">
         <v>438</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="C2" s="6">
+        <v>2</v>
+      </c>
+      <c r="D2" s="6">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
         <v>71</v>
-      </c>
-      <c r="E2" t="s">
-        <v>73</v>
       </c>
       <c r="F2" t="s">
         <v>73</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" t="s">
+        <v>73</v>
+      </c>
+      <c r="H2" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="I2" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="J2" s="7" t="s">
         <v>435</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="K2" s="7" t="s">
         <v>436</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>177</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>83</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>98</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>180</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>85</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>91</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>93</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
         <v>100</v>
       </c>
-      <c r="U2" s="6" t="s">
+      <c r="V2" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="V2" s="6" t="s">
+      <c r="W2" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="W2" t="s">
+      <c r="X2" t="s">
         <v>102</v>
       </c>
-      <c r="X2" t="s">
+      <c r="Y2" t="s">
         <v>105</v>
       </c>
-      <c r="Y2" s="6" t="s">
+      <c r="Z2" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="Z2" t="s">
+      <c r="AA2" t="s">
         <v>109</v>
       </c>
-      <c r="AA2" s="6" t="s">
+      <c r="AB2" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="AB2">
+      <c r="AC2">
         <v>5</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AD2" t="s">
         <v>111</v>
       </c>
-      <c r="AD2" t="s">
+      <c r="AE2" t="s">
         <v>176</v>
       </c>
-      <c r="AE2" t="s">
+      <c r="AF2" t="s">
         <v>182</v>
       </c>
-      <c r="AF2" s="9" t="s">
+      <c r="AG2" s="9" t="s">
         <v>203</v>
       </c>
     </row>
@@ -4763,29 +4772,30 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B43B544E-637D-4FD8-A2B1-2145904BBFF0}">
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:W2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.7109375" customWidth="1"/>
-    <col min="8" max="8" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" customWidth="1"/>
-    <col min="16" max="16" width="17.140625" customWidth="1"/>
-    <col min="17" max="17" width="16" customWidth="1"/>
-    <col min="20" max="20" width="17.7109375" customWidth="1"/>
-    <col min="21" max="21" width="12.85546875" customWidth="1"/>
-    <col min="22" max="22" width="15.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.7109375" customWidth="1"/>
+    <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.5703125" customWidth="1"/>
+    <col min="17" max="17" width="17.140625" customWidth="1"/>
+    <col min="18" max="18" width="16" customWidth="1"/>
+    <col min="21" max="21" width="17.7109375" customWidth="1"/>
+    <col min="22" max="22" width="12.85546875" customWidth="1"/>
+    <col min="23" max="23" width="15.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -4796,64 +4806,67 @@
         <v>69</v>
       </c>
       <c r="D1" t="s">
+        <v>441</v>
+      </c>
+      <c r="E1" t="s">
         <v>70</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>72</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>81</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>101</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>74</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>75</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>76</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>77</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>78</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>79</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>80</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>84</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>127</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>92</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>110</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>107</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>104</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>84</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>223</v>
       </c>
@@ -4864,55 +4877,58 @@
       <c r="C2" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="6">
+        <v>3</v>
+      </c>
+      <c r="E2" t="s">
         <v>86</v>
-      </c>
-      <c r="E2" t="s">
-        <v>73</v>
       </c>
       <c r="F2" t="s">
         <v>73</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" t="s">
+        <v>73</v>
+      </c>
+      <c r="H2" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="I2" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="J2" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="K2" s="7" t="s">
         <v>184</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>89</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>87</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>88</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>176</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>93</v>
       </c>
-      <c r="R2" s="6" t="s">
+      <c r="S2" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="S2" s="6" t="s">
+      <c r="T2" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
         <v>186</v>
       </c>
-      <c r="U2" t="s">
+      <c r="V2" t="s">
         <v>188</v>
       </c>
-      <c r="V2" t="s">
+      <c r="W2" t="s">
         <v>98</v>
       </c>
     </row>
@@ -5696,7 +5712,7 @@
       </c>
       <c r="B2" s="8" t="str">
         <f ca="1">TEXT(TODAY(), "DD/MM/YYYY")</f>
-        <v>04/06/2025</v>
+        <v>09/06/2025</v>
       </c>
       <c r="C2" t="s">
         <v>417</v>

</xml_diff>

<commit_message>
Change in Add medication
</commit_message>
<xml_diff>
--- a/ExcelFiles/PatientSummary.xlsx
+++ b/ExcelFiles/PatientSummary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Riomed\Cellma4ClinicalAuto2\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F0575D3-1E3C-4F9B-A3AF-139E934B1A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CACC224-14AA-422B-BD52-2CF688CF12E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loginDetails" sheetId="2" r:id="rId1"/>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="947" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="442">
   <si>
     <t>username</t>
   </si>
@@ -4066,11 +4066,11 @@
       <c r="B2" t="s">
         <v>438</v>
       </c>
-      <c r="C2" s="6">
-        <v>2</v>
-      </c>
-      <c r="D2" s="6">
-        <v>2</v>
+      <c r="C2" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>82</v>
       </c>
       <c r="E2" t="s">
         <v>71</v>
@@ -4877,8 +4877,8 @@
       <c r="C2" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="D2" s="6">
-        <v>3</v>
+      <c r="D2" s="6" t="s">
+        <v>113</v>
       </c>
       <c r="E2" t="s">
         <v>86</v>

</xml_diff>

<commit_message>
Added Devices, Medication Administration, Tests and Tool Categories
</commit_message>
<xml_diff>
--- a/ExcelFiles/PatientSummary.xlsx
+++ b/ExcelFiles/PatientSummary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Riomed\Cellma4ClinicalAuto2\ExcelFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Riomed\Cellma4ClinicalAuto\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69538DD9-19D1-43DF-B65C-6291795EB876}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93063035-C3AC-415E-8615-134F10C01031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-21600" windowWidth="19410" windowHeight="20985" firstSheet="62" activeTab="67" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loginDetails" sheetId="2" r:id="rId1"/>
@@ -74,6 +74,13 @@
     <sheet name="DeleteCarePlan" sheetId="59" r:id="rId59"/>
     <sheet name="Alerts" sheetId="60" r:id="rId60"/>
     <sheet name="DeleteInvestigation" sheetId="62" r:id="rId61"/>
+    <sheet name="DevicePatientDetails" sheetId="63" r:id="rId62"/>
+    <sheet name="AddDevice" sheetId="64" r:id="rId63"/>
+    <sheet name="EditDevice" sheetId="65" r:id="rId64"/>
+    <sheet name="AddTest" sheetId="66" r:id="rId65"/>
+    <sheet name="EditTest" sheetId="67" r:id="rId66"/>
+    <sheet name="AddTool" sheetId="68" r:id="rId67"/>
+    <sheet name="EditTool" sheetId="69" r:id="rId68"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -96,7 +103,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1228" uniqueCount="610">
   <si>
     <t>username</t>
   </si>
@@ -1419,6 +1426,513 @@
   </si>
   <si>
     <t>Knee Arthroplasty</t>
+  </si>
+  <si>
+    <t>AkaliA</t>
+  </si>
+  <si>
+    <t>Riomedtest</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>08/09/2024</t>
+  </si>
+  <si>
+    <t>dev_name</t>
+  </si>
+  <si>
+    <t>dev_type</t>
+  </si>
+  <si>
+    <t>dev_procedure_name</t>
+  </si>
+  <si>
+    <t>dev_manufacturer</t>
+  </si>
+  <si>
+    <t>dev_expiry_date</t>
+  </si>
+  <si>
+    <t>ded_type</t>
+  </si>
+  <si>
+    <t>ded_type_entry</t>
+  </si>
+  <si>
+    <t>ded_internal_external</t>
+  </si>
+  <si>
+    <t>ded_internal_external_entry</t>
+  </si>
+  <si>
+    <t>ded_laterality</t>
+  </si>
+  <si>
+    <t>ded_laterality_entry</t>
+  </si>
+  <si>
+    <t>ded_notes</t>
+  </si>
+  <si>
+    <t>ded_status</t>
+  </si>
+  <si>
+    <t>ded_status_entry</t>
+  </si>
+  <si>
+    <t>dev_serial_number</t>
+  </si>
+  <si>
+    <t>Cochlear Osia OSI200</t>
+  </si>
+  <si>
+    <t>Device</t>
+  </si>
+  <si>
+    <t>Cochlear Implantation</t>
+  </si>
+  <si>
+    <t>Cochlear</t>
+  </si>
+  <si>
+    <t>28/02/2025</t>
+  </si>
+  <si>
+    <t>Internal</t>
+  </si>
+  <si>
+    <t>Device added</t>
+  </si>
+  <si>
+    <t>Implanted</t>
+  </si>
+  <si>
+    <t>913748362</t>
+  </si>
+  <si>
+    <t>dev_deleted_reason</t>
+  </si>
+  <si>
+    <t>dev_ordering_status</t>
+  </si>
+  <si>
+    <t>Tool</t>
+  </si>
+  <si>
+    <t>SA Company</t>
+  </si>
+  <si>
+    <t>Device deleted</t>
+  </si>
+  <si>
+    <t>31/03/2025</t>
+  </si>
+  <si>
+    <t>First Stage</t>
+  </si>
+  <si>
+    <t>External</t>
+  </si>
+  <si>
+    <t>Device edited</t>
+  </si>
+  <si>
+    <t>awaitingapproval</t>
+  </si>
+  <si>
+    <t>pat_sex_at_birth</t>
+  </si>
+  <si>
+    <t>pattes_tests_question_que_name</t>
+  </si>
+  <si>
+    <t>pattes_answer_0</t>
+  </si>
+  <si>
+    <t>pattes_answer_1</t>
+  </si>
+  <si>
+    <t>pattes_answer_2</t>
+  </si>
+  <si>
+    <t>pattes_answer_3</t>
+  </si>
+  <si>
+    <t>pattes_answer_4</t>
+  </si>
+  <si>
+    <t>pattes_answer_5</t>
+  </si>
+  <si>
+    <t>pattes_answer_6</t>
+  </si>
+  <si>
+    <t>pattes_answer_7</t>
+  </si>
+  <si>
+    <t>pattes_answer_8</t>
+  </si>
+  <si>
+    <t>pattes_notes</t>
+  </si>
+  <si>
+    <t>Pressure Ulcer Test</t>
+  </si>
+  <si>
+    <t>Completely Limited</t>
+  </si>
+  <si>
+    <t>Constantly Moist</t>
+  </si>
+  <si>
+    <t>Chairfast</t>
+  </si>
+  <si>
+    <t>Completely Immobile</t>
+  </si>
+  <si>
+    <t>Probably Inadequate</t>
+  </si>
+  <si>
+    <t>Potential Problem</t>
+  </si>
+  <si>
+    <t>Add Pressure Ulcer Test</t>
+  </si>
+  <si>
+    <t>Malnutrition universal screening Test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt;20 </t>
+  </si>
+  <si>
+    <t>&lt;5%</t>
+  </si>
+  <si>
+    <t>Add Malnutrition universal screening Test</t>
+  </si>
+  <si>
+    <t>Falls Risk Assessment Scale</t>
+  </si>
+  <si>
+    <t>None in the last 12 months</t>
+  </si>
+  <si>
+    <t>Not taking any of these</t>
+  </si>
+  <si>
+    <t>Does not appear to have any of these</t>
+  </si>
+  <si>
+    <t>AMTS 9-10 OR intact</t>
+  </si>
+  <si>
+    <t>Add Falls Risk Assessment Scale</t>
+  </si>
+  <si>
+    <t>PHQ-9</t>
+  </si>
+  <si>
+    <t>Not at all</t>
+  </si>
+  <si>
+    <t>Several days</t>
+  </si>
+  <si>
+    <t>More than half the days</t>
+  </si>
+  <si>
+    <t>Nearly every days</t>
+  </si>
+  <si>
+    <t>Add PHQ-9 Test</t>
+  </si>
+  <si>
+    <t>pattes_review_date</t>
+  </si>
+  <si>
+    <t>pattes_last_reviewed</t>
+  </si>
+  <si>
+    <t>Very Limited</t>
+  </si>
+  <si>
+    <t>Very Moist</t>
+  </si>
+  <si>
+    <t>Bedfast</t>
+  </si>
+  <si>
+    <t>Slightly Limited</t>
+  </si>
+  <si>
+    <t>Very Poor</t>
+  </si>
+  <si>
+    <t>No Apparent Problem</t>
+  </si>
+  <si>
+    <t>Edit Pressure Ulcer Test</t>
+  </si>
+  <si>
+    <t>04/04/2025</t>
+  </si>
+  <si>
+    <t>Delete Test</t>
+  </si>
+  <si>
+    <t>&lt;18.5</t>
+  </si>
+  <si>
+    <t>&gt;10%</t>
+  </si>
+  <si>
+    <t>Edit Malnutrition universal screening Test</t>
+  </si>
+  <si>
+    <t>One or more between 3 and 12 months ago</t>
+  </si>
+  <si>
+    <t>Taking one</t>
+  </si>
+  <si>
+    <t>Appears mildly affected by one or more</t>
+  </si>
+  <si>
+    <t>AMTS 7-8 OR mildy impaired</t>
+  </si>
+  <si>
+    <t>Edit Falls Risk Assessment Scale</t>
+  </si>
+  <si>
+    <t>Edit PHQ-9 Test</t>
+  </si>
+  <si>
+    <t>medadt_medication_status</t>
+  </si>
+  <si>
+    <t>given</t>
+  </si>
+  <si>
+    <t>medi_notes_hidden</t>
+  </si>
+  <si>
+    <t>thayne.auto</t>
+  </si>
+  <si>
+    <t>Thayne@2024</t>
+  </si>
+  <si>
+    <t>pattod_var_value_0</t>
+  </si>
+  <si>
+    <t>pattod_var_value_1</t>
+  </si>
+  <si>
+    <t>pattod_var_value_2</t>
+  </si>
+  <si>
+    <t>pattod_var_value_3</t>
+  </si>
+  <si>
+    <t>pattod_var_value_4</t>
+  </si>
+  <si>
+    <t>patto_notes</t>
+  </si>
+  <si>
+    <t>Audiogram Tool</t>
+  </si>
+  <si>
+    <t>DAS 28 Examination Tool</t>
+  </si>
+  <si>
+    <t>DAS Examination notes</t>
+  </si>
+  <si>
+    <t>33</t>
+  </si>
+  <si>
+    <t>87</t>
+  </si>
+  <si>
+    <t>pattom_notes</t>
+  </si>
+  <si>
+    <t>Patient marker functionality test</t>
+  </si>
+  <si>
+    <t>DAS28</t>
+  </si>
+  <si>
+    <t>clinicItem</t>
+  </si>
+  <si>
+    <t>09/05/2025</t>
+  </si>
+  <si>
+    <t>patto_review_date</t>
+  </si>
+  <si>
+    <t>patto_last_reviewed</t>
+  </si>
+  <si>
+    <t>Delete Tool</t>
+  </si>
+  <si>
+    <t>75</t>
+  </si>
+  <si>
+    <t>67</t>
+  </si>
+  <si>
+    <t>42</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>Edit tool test</t>
+  </si>
+  <si>
+    <t>DAS78</t>
+  </si>
+  <si>
+    <t>DAS 78 New tool</t>
+  </si>
+  <si>
+    <t>DAS 78 Examination Tool</t>
+  </si>
+  <si>
+    <t>Patient marker for DAS 78</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>DAS 78 Edit Tool</t>
+  </si>
+  <si>
+    <t>09/05/2026</t>
+  </si>
+  <si>
+    <t>VRA</t>
+  </si>
+  <si>
+    <t>Pure tone</t>
+  </si>
+  <si>
+    <t>Reliability Air Conduction</t>
+  </si>
+  <si>
+    <t>Headphones</t>
+  </si>
+  <si>
+    <t>Play Audiometry</t>
+  </si>
+  <si>
+    <t>Warble</t>
+  </si>
+  <si>
+    <t>Behavioural Observation Audiometry</t>
+  </si>
+  <si>
+    <t>Narrowband noise</t>
+  </si>
+  <si>
+    <t>Reliability Unaided Soundfield</t>
+  </si>
+  <si>
+    <t>Patient Response Button</t>
+  </si>
+  <si>
+    <t>White noise</t>
+  </si>
+  <si>
+    <t>Reliability Aided Soundfield</t>
+  </si>
+  <si>
+    <t>pattod_var_value_5</t>
+  </si>
+  <si>
+    <t>pattod_var_value_6</t>
+  </si>
+  <si>
+    <t>pattod_var_value_7</t>
+  </si>
+  <si>
+    <t>pattod_var_value_8</t>
+  </si>
+  <si>
+    <t>pattod_var_value_9</t>
+  </si>
+  <si>
+    <t>pattod_var_value_10</t>
+  </si>
+  <si>
+    <t>pattod_var_value_11</t>
+  </si>
+  <si>
+    <t>pattod_var_value_12</t>
+  </si>
+  <si>
+    <t>patto_notes_0</t>
+  </si>
+  <si>
+    <t>patto_notes_1</t>
+  </si>
+  <si>
+    <t>patto_notes_2</t>
+  </si>
+  <si>
+    <t>patto_notes_3</t>
+  </si>
+  <si>
+    <t>Notes on Air Conduction</t>
+  </si>
+  <si>
+    <t>Notes on Bone Conduction</t>
+  </si>
+  <si>
+    <t>Notes on Unaided Soundfield</t>
+  </si>
+  <si>
+    <t>Notes on Aided Soundfield</t>
+  </si>
+  <si>
+    <t>Reliability Bone Conduction</t>
+  </si>
+  <si>
+    <t>Edit  Air Conduction</t>
+  </si>
+  <si>
+    <t>Edit Bone Conduction</t>
+  </si>
+  <si>
+    <t>Edit Unaided Soundfield</t>
+  </si>
+  <si>
+    <t>Edit Aided Soundfield</t>
+  </si>
+  <si>
+    <t>Reliability Air Conduction Edited</t>
+  </si>
+  <si>
+    <t>Speaker</t>
+  </si>
+  <si>
+    <t>Reliability Bone Conduction Edited</t>
+  </si>
+  <si>
+    <t>Reliability Unaided Soundfield Edited</t>
+  </si>
+  <si>
+    <t>Reliability Aided Soundfield Edited</t>
   </si>
 </sst>
 </file>
@@ -1428,7 +1942,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\/mm\/yyyy"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1449,6 +1963,12 @@
       <color rgb="FF000000"/>
       <name val="Consolas"/>
       <family val="3"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1779,14 +2299,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DE4FC9F-2982-4FD6-8BD6-4330FF8DA2DE}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.140625" customWidth="1"/>
-    <col min="2" max="2" width="17.5703125" customWidth="1"/>
+    <col min="1" max="1" width="21.1796875" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1794,26 +2314,35 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>538</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>283</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B3" s="1" t="s">
         <v>437</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>375</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>376</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{0C05B6B9-5554-4DE8-9F6A-6002C7FF4022}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{03C77328-BA61-4FC6-A325-FBFA15AC6C52}"/>
+    <hyperlink ref="B3" r:id="rId1" xr:uid="{0C05B6B9-5554-4DE8-9F6A-6002C7FF4022}"/>
+    <hyperlink ref="B4" r:id="rId2" xr:uid="{03C77328-BA61-4FC6-A325-FBFA15AC6C52}"/>
+    <hyperlink ref="B2" r:id="rId3" xr:uid="{93D54D70-B776-425E-A1AB-5F66698FEC3B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1822,13 +2351,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5682E5CD-63B5-4779-9930-5C9E9312DCA8}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -1836,7 +2365,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>200</v>
       </c>
@@ -1852,17 +2381,17 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7070D364-07A9-4E81-9AAD-6D06CFE64A7E}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" customWidth="1"/>
-    <col min="2" max="2" width="23.85546875" customWidth="1"/>
-    <col min="3" max="3" width="20.7109375" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" customWidth="1"/>
+    <col min="1" max="1" width="26.453125" customWidth="1"/>
+    <col min="2" max="2" width="23.81640625" customWidth="1"/>
+    <col min="3" max="3" width="20.7265625" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" customWidth="1"/>
     <col min="5" max="5" width="19" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.85546875" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -1882,7 +2411,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>222</v>
       </c>
@@ -1911,15 +2440,15 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4C74051-56F8-4BE3-95DE-85BE5950FD64}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.1796875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -1936,7 +2465,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>222</v>
       </c>
@@ -1961,13 +2490,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69EDCE76-70F4-4473-B92F-8913C9A903B8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.42578125" customWidth="1"/>
-    <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.453125" customWidth="1"/>
+    <col min="2" max="2" width="15.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -1978,7 +2507,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>222</v>
       </c>
@@ -1997,17 +2526,17 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F50D2E72-168F-40F2-B5D3-65D8E679AC63}">
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="6" width="19.5703125" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="6" width="19.54296875" customWidth="1"/>
     <col min="7" max="7" width="17" customWidth="1"/>
-    <col min="8" max="8" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="26.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -2036,7 +2565,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>149</v>
       </c>
@@ -2073,20 +2602,20 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8027F072-5B7F-474B-8D83-79953C31361B}">
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.7265625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.140625" customWidth="1"/>
-    <col min="8" max="8" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.1796875" customWidth="1"/>
+    <col min="8" max="8" width="16.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="26.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -2115,7 +2644,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>149</v>
       </c>
@@ -2152,13 +2681,13 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{008CC7AC-AB6D-4187-B6A0-1158E613B828}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.28515625" customWidth="1"/>
-    <col min="2" max="2" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="26.26953125" customWidth="1"/>
+    <col min="2" max="2" width="18.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -2166,7 +2695,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>150</v>
       </c>
@@ -2182,19 +2711,19 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{094FA7C7-2F9F-473D-A811-B803747DC0A3}">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.85546875" customWidth="1"/>
-    <col min="5" max="5" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.140625" customWidth="1"/>
-    <col min="9" max="11" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.42578125" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.81640625" customWidth="1"/>
+    <col min="5" max="5" width="20.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.1796875" customWidth="1"/>
+    <col min="9" max="11" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -2238,7 +2767,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>134</v>
       </c>
@@ -2288,19 +2817,19 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92D95DB8-7522-4276-90BD-0BAB60F0AAE6}">
   <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.85546875" customWidth="1"/>
-    <col min="5" max="5" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="32.85546875" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.81640625" customWidth="1"/>
+    <col min="5" max="5" width="20.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="32.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -2338,7 +2867,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>134</v>
       </c>
@@ -2381,13 +2910,13 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70DCF4C9-25DB-44CD-A95D-99E79260CBAB}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.28515625" customWidth="1"/>
-    <col min="2" max="2" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="26.26953125" customWidth="1"/>
+    <col min="2" max="2" width="18.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -2395,7 +2924,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>135</v>
       </c>
@@ -2410,16 +2939,61 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFF0DF87-67F2-4E87-A7EE-C4365800D834}">
-  <dimension ref="A1:AV2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AW2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" customWidth="1"/>
-    <col min="7" max="7" width="16.42578125" customWidth="1"/>
-    <col min="9" max="9" width="11.140625" customWidth="1"/>
+    <col min="1" max="1" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.90625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.6328125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="19.90625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="24.90625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="24.54296875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="12" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="23.54296875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="20.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="8.26953125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="28.36328125" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="18.08984375" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="16.6328125" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="30.54296875" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="27.54296875" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="16.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:49" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -2445,127 +3019,130 @@
         <v>9</v>
       </c>
       <c r="I1" t="s">
+        <v>479</v>
+      </c>
+      <c r="J1" t="s">
         <v>10</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>11</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>12</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>13</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>14</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>15</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>16</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>17</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>18</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>19</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>20</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>21</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>22</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>23</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>24</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>25</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>26</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>27</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>28</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>29</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AD1" t="s">
         <v>30</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AE1" t="s">
         <v>31</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AF1" t="s">
         <v>32</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AG1" t="s">
         <v>33</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AH1" t="s">
         <v>34</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AI1" t="s">
         <v>35</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AJ1" t="s">
         <v>36</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AK1" t="s">
         <v>37</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AL1" t="s">
         <v>38</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AM1" t="s">
         <v>39</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AN1" t="s">
         <v>40</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AO1" t="s">
         <v>41</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AP1" t="s">
         <v>42</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AQ1" t="s">
         <v>43</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AR1" t="s">
         <v>44</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AS1" t="s">
         <v>45</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AT1" t="s">
         <v>46</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AU1" t="s">
         <v>47</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AV1" t="s">
         <v>48</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AW1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:48" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:49" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B2" s="3" t="s">
         <v>378</v>
       </c>
@@ -2581,76 +3158,79 @@
       <c r="H2" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="J2" s="4" t="s">
         <v>434</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="M2" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="O2" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="Q2" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="S2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="T2" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="U2" s="3" t="s">
+      <c r="V2" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="V2" s="3" t="s">
+      <c r="W2" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="W2" s="2">
+      <c r="X2" s="2">
         <v>0</v>
       </c>
-      <c r="X2" s="3" t="s">
+      <c r="Y2" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="Y2" s="2">
+      <c r="Z2" s="2">
         <v>0</v>
       </c>
-      <c r="Z2" s="3" t="s">
+      <c r="AA2" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="AB2" s="5" t="s">
+      <c r="AC2" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="AI2" s="3" t="s">
+      <c r="AJ2" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="AJ2" s="3" t="s">
+      <c r="AK2" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="AM2" s="3" t="s">
+      <c r="AN2" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="AO2" t="s">
+      <c r="AP2" t="s">
         <v>60</v>
       </c>
-      <c r="AQ2" s="3" t="s">
+      <c r="AR2" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="AR2" s="2" t="s">
+      <c r="AS2" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="AU2" s="3" t="s">
+      <c r="AV2" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="AV2" s="3" t="s">
+      <c r="AW2" s="3" t="s">
         <v>66</v>
       </c>
     </row>
@@ -2662,17 +3242,17 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{073326C8-FACB-4B5B-B1CF-ABFED8B93DBE}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.42578125" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.453125" customWidth="1"/>
+    <col min="5" max="5" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -2692,7 +3272,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>171</v>
       </c>
@@ -2720,17 +3300,17 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F596452A-5694-4E32-87F2-C18569884D3B}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.42578125" customWidth="1"/>
-    <col min="5" max="5" width="21.7109375" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="2" max="2" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.453125" customWidth="1"/>
+    <col min="5" max="5" width="21.7265625" customWidth="1"/>
+    <col min="6" max="6" width="14.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -2750,7 +3330,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>171</v>
       </c>
@@ -2778,14 +3358,14 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8852AC2C-7F1F-45E0-AA81-1C0AC8298BDB}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="2" max="2" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -2796,7 +3376,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>171</v>
       </c>
@@ -2815,20 +3395,20 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C664057-036F-45F9-BB17-F131467544E4}">
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.42578125" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.453125" customWidth="1"/>
+    <col min="5" max="5" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.81640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17" customWidth="1"/>
-    <col min="8" max="8" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -2854,7 +3434,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>194</v>
       </c>
@@ -2866,7 +3446,7 @@
       </c>
       <c r="D2" s="7" t="str">
         <f ca="1">TEXT(TODAY(), "DD/MM/YYYY")</f>
-        <v>04/06/2025</v>
+        <v>17/06/2025</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>198</v>
@@ -2890,19 +3470,19 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DE09E9A-9C0C-49EF-BEE4-12AF4C853339}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.42578125" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.28515625" customWidth="1"/>
-    <col min="8" max="8" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.453125" customWidth="1"/>
+    <col min="5" max="5" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.26953125" customWidth="1"/>
+    <col min="8" max="8" width="13.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -2928,7 +3508,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>194</v>
       </c>
@@ -2940,7 +3520,7 @@
       </c>
       <c r="D2" s="7" t="str">
         <f ca="1">TEXT(TODAY(), "DD/MM/YYYY")</f>
-        <v>04/06/2025</v>
+        <v>17/06/2025</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>199</v>
@@ -2963,14 +3543,14 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F4129C8-341D-4D38-92A2-748311EBE13A}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="2" max="2" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -2981,7 +3561,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>194</v>
       </c>
@@ -3000,23 +3580,23 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9AC72BC-1449-4578-8E57-945920649F3D}">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="1"/>
-    <col min="2" max="2" width="31.7109375" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="2" max="2" width="31.7265625" customWidth="1"/>
     <col min="3" max="3" width="21" customWidth="1"/>
-    <col min="4" max="6" width="17.42578125" customWidth="1"/>
-    <col min="7" max="7" width="22.28515625" customWidth="1"/>
-    <col min="8" max="8" width="20.85546875" customWidth="1"/>
-    <col min="9" max="9" width="15.7109375" customWidth="1"/>
-    <col min="10" max="10" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.7109375" customWidth="1"/>
-    <col min="12" max="12" width="17.42578125" customWidth="1"/>
+    <col min="4" max="6" width="17.453125" customWidth="1"/>
+    <col min="7" max="7" width="22.26953125" customWidth="1"/>
+    <col min="8" max="8" width="20.81640625" customWidth="1"/>
+    <col min="9" max="9" width="15.7265625" customWidth="1"/>
+    <col min="10" max="10" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.7265625" customWidth="1"/>
+    <col min="12" max="12" width="17.453125" customWidth="1"/>
     <col min="13" max="13" width="15" customWidth="1"/>
-    <col min="14" max="14" width="12.85546875" customWidth="1"/>
+    <col min="14" max="14" width="12.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -3060,7 +3640,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>213</v>
       </c>
@@ -3112,19 +3692,19 @@
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80A773DA-484D-48A0-B5A2-743931447EDE}">
   <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" customWidth="1"/>
+    <col min="4" max="4" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.81640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17" customWidth="1"/>
-    <col min="7" max="7" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -3162,7 +3742,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>213</v>
       </c>
@@ -3171,7 +3751,7 @@
       </c>
       <c r="C2" s="7">
         <f ca="1">TODAY()</f>
-        <v>45812</v>
+        <v>45825</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>103</v>
@@ -3209,14 +3789,14 @@
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3A63575-EEB1-470D-A815-33D356B026F2}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" customWidth="1"/>
+    <col min="3" max="3" width="18.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -3227,7 +3807,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>213</v>
       </c>
@@ -3246,12 +3826,12 @@
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A6156A5-E27D-4C56-9CFB-F9306D57D7B5}">
   <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="7" max="7" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -3292,7 +3872,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>232</v>
       </c>
@@ -3341,7 +3921,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3350,24 +3930,24 @@
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DDECB00-706E-4E8F-A123-3F48B34B46C2}">
   <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="41.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.7109375" customWidth="1"/>
-    <col min="5" max="5" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="26.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.5703125" style="11" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.7109375" style="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.85546875" style="11" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="41.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.7265625" customWidth="1"/>
+    <col min="5" max="5" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.1796875" style="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.54296875" style="11" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.7265625" style="11" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.81640625" style="11" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="16" style="11" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.453125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="22" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -3408,7 +3988,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>232</v>
       </c>
@@ -3457,13 +4037,13 @@
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAB902D2-410D-470A-9E88-FE4AC8B16D55}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -3471,7 +4051,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>233</v>
       </c>
@@ -3487,22 +4067,22 @@
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89AB0309-4D83-402B-A384-3BBD8F0E5F31}">
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
-    <col min="2" max="2" width="23.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.81640625" customWidth="1"/>
+    <col min="2" max="2" width="23.81640625" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="16.5703125" customWidth="1"/>
-    <col min="5" max="5" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="26.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.54296875" customWidth="1"/>
+    <col min="5" max="5" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.26953125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -3537,7 +4117,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>247</v>
       </c>
@@ -3580,22 +4160,22 @@
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B38BF4A6-8DEB-41FA-A7FD-F0100AB3FE2C}">
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
-    <col min="2" max="2" width="23.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.81640625" customWidth="1"/>
+    <col min="2" max="2" width="23.81640625" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="16.5703125" customWidth="1"/>
-    <col min="5" max="5" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="26.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.54296875" customWidth="1"/>
+    <col min="5" max="5" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.26953125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -3630,7 +4210,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>247</v>
       </c>
@@ -3673,13 +4253,13 @@
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC23809B-2D36-41E4-A3B9-65D4308A6DCA}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -3687,7 +4267,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>439</v>
       </c>
@@ -3703,17 +4283,17 @@
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FF9792A-063B-40AF-9553-C8061AFC39D0}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.5703125" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.54296875" customWidth="1"/>
     <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -3733,7 +4313,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>260</v>
       </c>
@@ -3761,15 +4341,15 @@
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B8717C7-2D4F-48DD-A7CA-84784DCBB919}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.140625" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.1796875" customWidth="1"/>
+    <col min="4" max="4" width="16.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -3783,7 +4363,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>260</v>
       </c>
@@ -3805,13 +4385,13 @@
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BF370ED-86AA-4D7E-B092-14AB12F95410}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.28515625" customWidth="1"/>
-    <col min="2" max="2" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="26.26953125" customWidth="1"/>
+    <col min="2" max="2" width="18.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -3819,7 +4399,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>260</v>
       </c>
@@ -3835,15 +4415,15 @@
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28DAC4B0-6F7A-40C4-8629-2F293F19EE6C}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" customWidth="1"/>
-    <col min="4" max="4" width="22.140625" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" customWidth="1"/>
+    <col min="4" max="4" width="22.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -3857,7 +4437,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>269</v>
       </c>
@@ -3879,15 +4459,15 @@
 <file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4EF1174-5299-4F4F-A888-C15D55804D2F}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" customWidth="1"/>
-    <col min="4" max="4" width="22.140625" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" customWidth="1"/>
+    <col min="4" max="4" width="22.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -3901,7 +4481,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>269</v>
       </c>
@@ -3922,40 +4502,44 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DD9439C-0973-45AC-88BC-21584AF7E144}">
-  <dimension ref="A1:AF2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AG2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.42578125" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="8" width="13.7109375" customWidth="1"/>
-    <col min="9" max="9" width="11.85546875" customWidth="1"/>
-    <col min="10" max="10" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.42578125" customWidth="1"/>
-    <col min="12" max="12" width="12.5703125" customWidth="1"/>
-    <col min="13" max="13" width="17" customWidth="1"/>
-    <col min="14" max="16" width="15.5703125" customWidth="1"/>
-    <col min="17" max="17" width="12.85546875" customWidth="1"/>
-    <col min="18" max="18" width="16.5703125" customWidth="1"/>
-    <col min="19" max="20" width="16" customWidth="1"/>
-    <col min="21" max="21" width="13.140625" customWidth="1"/>
-    <col min="22" max="22" width="21" customWidth="1"/>
-    <col min="23" max="23" width="13.140625" customWidth="1"/>
-    <col min="24" max="24" width="17.7109375" customWidth="1"/>
-    <col min="25" max="25" width="13.85546875" customWidth="1"/>
-    <col min="26" max="26" width="12.28515625" customWidth="1"/>
-    <col min="27" max="27" width="15.140625" customWidth="1"/>
-    <col min="28" max="28" width="28.42578125" customWidth="1"/>
-    <col min="29" max="29" width="14.85546875" customWidth="1"/>
-    <col min="30" max="30" width="17.140625" customWidth="1"/>
-    <col min="31" max="31" width="27.140625" customWidth="1"/>
-    <col min="32" max="32" width="12.85546875" customWidth="1"/>
+    <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="23.81640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="27.90625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="32.26953125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="25.7265625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="23.453125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="21.26953125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="23.453125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="21.90625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="14.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -4005,7 +4589,7 @@
         <v>179</v>
       </c>
       <c r="Q1" t="s">
-        <v>84</v>
+        <v>537</v>
       </c>
       <c r="R1" t="s">
         <v>90</v>
@@ -4052,8 +4636,11 @@
       <c r="AF1" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG1" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>223</v>
       </c>
@@ -4143,6 +4730,9 @@
       </c>
       <c r="AF2" s="9" t="s">
         <v>203</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>536</v>
       </c>
     </row>
   </sheetData>
@@ -4153,14 +4743,14 @@
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF82F3D0-82CD-49AF-BA0A-7CEE53FBA6AC}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="28.140625" customWidth="1"/>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="28.1796875" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -4171,7 +4761,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>269</v>
       </c>
@@ -4190,15 +4780,15 @@
 <file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFEABC41-711E-4537-AE0B-FD45295FCA16}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" customWidth="1"/>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" customWidth="1"/>
-    <col min="4" max="4" width="22.140625" customWidth="1"/>
+    <col min="1" max="1" width="19.26953125" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" customWidth="1"/>
+    <col min="4" max="4" width="22.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -4212,7 +4802,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>274</v>
       </c>
@@ -4234,15 +4824,15 @@
 <file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BCAE196-8758-4745-8A92-E19A1A017AF5}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" customWidth="1"/>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" customWidth="1"/>
-    <col min="4" max="4" width="22.140625" customWidth="1"/>
+    <col min="1" max="1" width="19.26953125" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" customWidth="1"/>
+    <col min="4" max="4" width="22.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -4256,7 +4846,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>274</v>
       </c>
@@ -4278,14 +4868,14 @@
 <file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA3F2689-A05C-47BB-9880-495021A0BDBF}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="28.140625" customWidth="1"/>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="28.1796875" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -4296,7 +4886,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>270</v>
       </c>
@@ -4315,14 +4905,14 @@
 <file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{025D1112-B23A-48F4-BA89-51264C4515AC}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.28515625" customWidth="1"/>
-    <col min="3" max="4" width="16.7109375" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.26953125" customWidth="1"/>
+    <col min="3" max="4" width="16.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -4336,7 +4926,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>279</v>
       </c>
@@ -4358,14 +4948,14 @@
 <file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD2F5B74-CFA6-4CF1-AE93-E1D942D7EC4C}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.28515625" customWidth="1"/>
-    <col min="3" max="4" width="16.7109375" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.26953125" customWidth="1"/>
+    <col min="3" max="4" width="16.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -4379,7 +4969,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>279</v>
       </c>
@@ -4401,14 +4991,14 @@
 <file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{206A2E86-90FC-4080-A7DC-7A2B6DBA9D36}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="28.140625" customWidth="1"/>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="28.1796875" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -4419,7 +5009,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>279</v>
       </c>
@@ -4438,18 +5028,18 @@
 <file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA6646E2-86C9-4AB0-83E3-F184F5C30E9A}">
   <dimension ref="A1:Q2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="16.7109375" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="16.7265625" customWidth="1"/>
+    <col min="5" max="5" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="15" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -4502,7 +5092,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>287</v>
       </c>
@@ -4560,19 +5150,19 @@
 <file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{132C5A93-3712-47E8-A929-16017ECD465E}">
   <dimension ref="A1:U2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="16.7109375" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="16.7265625" customWidth="1"/>
+    <col min="5" max="5" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="15" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="23" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -4637,7 +5227,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>287</v>
       </c>
@@ -4707,16 +5297,16 @@
 <file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1194F774-EACE-44AC-9C8A-A1CC70FE36E1}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="1"/>
-    <col min="2" max="3" width="25.5703125" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="2" max="3" width="25.54296875" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="20.28515625" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.26953125" customWidth="1"/>
+    <col min="6" max="6" width="14.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -4736,7 +5326,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>324</v>
       </c>
@@ -4764,28 +5354,28 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B43B544E-637D-4FD8-A2B1-2145904BBFF0}">
   <dimension ref="A1:V2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.7109375" customWidth="1"/>
-    <col min="8" max="8" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" customWidth="1"/>
-    <col min="16" max="16" width="17.140625" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.7265625" customWidth="1"/>
+    <col min="8" max="8" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.54296875" customWidth="1"/>
+    <col min="16" max="16" width="17.1796875" customWidth="1"/>
     <col min="17" max="17" width="16" customWidth="1"/>
-    <col min="20" max="20" width="17.7109375" customWidth="1"/>
-    <col min="21" max="21" width="12.85546875" customWidth="1"/>
-    <col min="22" max="22" width="15.5703125" customWidth="1"/>
+    <col min="20" max="20" width="17.7265625" customWidth="1"/>
+    <col min="21" max="21" width="12.81640625" customWidth="1"/>
+    <col min="22" max="22" width="15.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -4853,7 +5443,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>223</v>
       </c>
@@ -4924,16 +5514,16 @@
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01C7CE86-1D30-42A6-BFFE-DD7CB531D10C}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="1"/>
-    <col min="2" max="3" width="25.5703125" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="2" max="3" width="25.54296875" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="19.28515625" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.26953125" customWidth="1"/>
+    <col min="6" max="6" width="14.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -4953,7 +5543,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>324</v>
       </c>
@@ -4981,13 +5571,13 @@
 <file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06A0A6C0-CF2F-48B8-BAC5-F3E5690001A5}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="1"/>
-    <col min="2" max="2" width="25.5703125" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="2" max="2" width="25.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -4995,7 +5585,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>324</v>
       </c>
@@ -5011,15 +5601,15 @@
 <file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{120AD279-3012-4840-AF87-588B2BE3B2AA}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -5033,7 +5623,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>333</v>
       </c>
@@ -5056,15 +5646,15 @@
 <file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C038ED2-3C9D-4D5B-A9F6-773661E9B6A6}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.1796875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -5078,7 +5668,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>333</v>
       </c>
@@ -5100,14 +5690,14 @@
 <file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{796CA3FD-2DF2-4849-A599-7F2B1477C186}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -5118,7 +5708,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>333</v>
       </c>
@@ -5137,23 +5727,23 @@
 <file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C6C2239-2180-4B9C-B8A1-E16F3FCE77A5}">
   <dimension ref="A1:O2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="14.28515625" customWidth="1"/>
-    <col min="6" max="6" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="14.26953125" customWidth="1"/>
+    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.453125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.26953125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="21" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>338</v>
       </c>
@@ -5200,7 +5790,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>353</v>
       </c>
@@ -5255,20 +5845,20 @@
 <file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B730A7AF-1268-4970-A808-63C4CFDE9D42}">
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.453125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.26953125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="21" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>365</v>
       </c>
@@ -5303,7 +5893,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" s="10" t="s">
         <v>368</v>
       </c>
@@ -5346,24 +5936,24 @@
 <file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DCFF350-CD6D-4EA3-AD07-F7835D15A2E0}">
   <dimension ref="A1:P2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.28515625" customWidth="1"/>
-    <col min="2" max="2" width="17.42578125" customWidth="1"/>
-    <col min="3" max="3" width="23.140625" customWidth="1"/>
-    <col min="4" max="4" width="14.7109375" customWidth="1"/>
-    <col min="5" max="5" width="21.7109375" customWidth="1"/>
+    <col min="1" max="1" width="15.26953125" customWidth="1"/>
+    <col min="2" max="2" width="17.453125" customWidth="1"/>
+    <col min="3" max="3" width="23.1796875" customWidth="1"/>
+    <col min="4" max="4" width="14.7265625" customWidth="1"/>
+    <col min="5" max="5" width="21.7265625" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="15.85546875" customWidth="1"/>
-    <col min="8" max="8" width="20.5703125" customWidth="1"/>
-    <col min="9" max="10" width="19.7109375" customWidth="1"/>
+    <col min="7" max="7" width="15.81640625" customWidth="1"/>
+    <col min="8" max="8" width="20.54296875" customWidth="1"/>
+    <col min="9" max="10" width="19.7265625" customWidth="1"/>
     <col min="12" max="12" width="23" customWidth="1"/>
-    <col min="13" max="13" width="20.5703125" customWidth="1"/>
-    <col min="14" max="14" width="11.7109375" customWidth="1"/>
-    <col min="15" max="15" width="21.140625" customWidth="1"/>
+    <col min="13" max="13" width="20.54296875" customWidth="1"/>
+    <col min="14" max="14" width="11.7265625" customWidth="1"/>
+    <col min="15" max="15" width="21.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -5410,7 +6000,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>405</v>
       </c>
@@ -5468,24 +6058,24 @@
 <file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{019DB1EE-87BC-46CC-8969-22DDA41D9703}">
   <dimension ref="A1:P2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.28515625" customWidth="1"/>
-    <col min="2" max="2" width="17.42578125" customWidth="1"/>
-    <col min="3" max="3" width="23.140625" customWidth="1"/>
-    <col min="4" max="4" width="14.7109375" customWidth="1"/>
-    <col min="5" max="5" width="21.7109375" customWidth="1"/>
+    <col min="1" max="1" width="15.26953125" customWidth="1"/>
+    <col min="2" max="2" width="17.453125" customWidth="1"/>
+    <col min="3" max="3" width="23.1796875" customWidth="1"/>
+    <col min="4" max="4" width="14.7265625" customWidth="1"/>
+    <col min="5" max="5" width="21.7265625" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="15.85546875" customWidth="1"/>
-    <col min="8" max="8" width="20.5703125" customWidth="1"/>
-    <col min="9" max="10" width="19.7109375" customWidth="1"/>
+    <col min="7" max="7" width="15.81640625" customWidth="1"/>
+    <col min="8" max="8" width="20.54296875" customWidth="1"/>
+    <col min="9" max="10" width="19.7265625" customWidth="1"/>
     <col min="12" max="12" width="23" customWidth="1"/>
-    <col min="13" max="13" width="20.5703125" customWidth="1"/>
-    <col min="14" max="14" width="11.7109375" customWidth="1"/>
-    <col min="15" max="15" width="21.140625" customWidth="1"/>
+    <col min="13" max="13" width="20.54296875" customWidth="1"/>
+    <col min="14" max="14" width="11.7265625" customWidth="1"/>
+    <col min="15" max="15" width="21.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -5532,7 +6122,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>405</v>
       </c>
@@ -5590,7 +6180,7 @@
 <file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{073EB301-EA84-4595-9FAF-2D4DB18F33CC}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5599,14 +6189,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3765FB4-F532-4FCF-A614-4266393F4C44}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -5617,7 +6207,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>223</v>
       </c>
@@ -5637,22 +6227,22 @@
 <file path=xl/worksheets/sheet60.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{292FBDAE-D596-4C82-A946-FDA545BEF94C}">
   <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.5703125" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" customWidth="1"/>
-    <col min="4" max="4" width="19.140625" customWidth="1"/>
-    <col min="5" max="5" width="12.42578125" customWidth="1"/>
-    <col min="6" max="6" width="16.42578125" customWidth="1"/>
-    <col min="7" max="7" width="11.85546875" customWidth="1"/>
-    <col min="8" max="8" width="13.5703125" customWidth="1"/>
-    <col min="9" max="9" width="11.7109375" customWidth="1"/>
-    <col min="10" max="10" width="13.28515625" customWidth="1"/>
-    <col min="11" max="11" width="18.28515625" customWidth="1"/>
+    <col min="1" max="1" width="20.54296875" customWidth="1"/>
+    <col min="2" max="2" width="18.26953125" customWidth="1"/>
+    <col min="3" max="3" width="14.1796875" customWidth="1"/>
+    <col min="4" max="4" width="19.1796875" customWidth="1"/>
+    <col min="5" max="5" width="12.453125" customWidth="1"/>
+    <col min="6" max="6" width="16.453125" customWidth="1"/>
+    <col min="7" max="7" width="11.81640625" customWidth="1"/>
+    <col min="8" max="8" width="13.54296875" customWidth="1"/>
+    <col min="9" max="9" width="11.7265625" customWidth="1"/>
+    <col min="10" max="10" width="13.26953125" customWidth="1"/>
+    <col min="11" max="11" width="18.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>411</v>
       </c>
@@ -5690,13 +6280,13 @@
         <v>429</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
         <v>427</v>
       </c>
       <c r="B2" s="8" t="str">
         <f ca="1">TEXT(TODAY(), "DD/MM/YYYY")</f>
-        <v>04/06/2025</v>
+        <v>17/06/2025</v>
       </c>
       <c r="C2" t="s">
         <v>417</v>
@@ -5734,18 +6324,18 @@
 <file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB9C9D7F-0AE8-4EC3-92AB-0B4F9C52B57D}">
   <dimension ref="A1:Q2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="16.7109375" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="16.7265625" customWidth="1"/>
+    <col min="5" max="5" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="15" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -5798,7 +6388,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>287</v>
       </c>
@@ -5854,10 +6444,1121 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{346D593C-0211-4209-AF2A-C9DAEA3833CA}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.453125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>444</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39C0FE73-9A12-4221-A381-CB00E26B6D80}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.90625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>445</v>
+      </c>
+      <c r="B1" t="s">
+        <v>446</v>
+      </c>
+      <c r="C1" t="s">
+        <v>447</v>
+      </c>
+      <c r="D1" t="s">
+        <v>448</v>
+      </c>
+      <c r="E1" t="s">
+        <v>449</v>
+      </c>
+      <c r="F1" t="s">
+        <v>450</v>
+      </c>
+      <c r="G1" t="s">
+        <v>451</v>
+      </c>
+      <c r="H1" t="s">
+        <v>452</v>
+      </c>
+      <c r="I1" t="s">
+        <v>453</v>
+      </c>
+      <c r="J1" t="s">
+        <v>454</v>
+      </c>
+      <c r="K1" t="s">
+        <v>455</v>
+      </c>
+      <c r="L1" t="s">
+        <v>456</v>
+      </c>
+      <c r="M1" t="s">
+        <v>457</v>
+      </c>
+      <c r="N1" t="s">
+        <v>458</v>
+      </c>
+      <c r="O1" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>460</v>
+      </c>
+      <c r="B2" t="s">
+        <v>461</v>
+      </c>
+      <c r="C2" t="s">
+        <v>462</v>
+      </c>
+      <c r="D2" t="s">
+        <v>463</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>464</v>
+      </c>
+      <c r="F2" t="str">
+        <f>LOWER(G2)</f>
+        <v>primary</v>
+      </c>
+      <c r="G2" t="s">
+        <v>212</v>
+      </c>
+      <c r="H2" t="str">
+        <f>LOWER(I2)</f>
+        <v>internal</v>
+      </c>
+      <c r="I2" t="s">
+        <v>465</v>
+      </c>
+      <c r="J2" t="str">
+        <f>LOWER(K2)</f>
+        <v>left</v>
+      </c>
+      <c r="K2" t="s">
+        <v>103</v>
+      </c>
+      <c r="L2" t="s">
+        <v>466</v>
+      </c>
+      <c r="M2" t="str">
+        <f>LOWER(N2)</f>
+        <v>implanted</v>
+      </c>
+      <c r="N2" t="s">
+        <v>467</v>
+      </c>
+      <c r="O2" s="6" t="s">
+        <v>468</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12B70FEE-6B1F-41AF-B992-BCB179E19A76}">
+  <dimension ref="A1:P2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="24.90625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>445</v>
+      </c>
+      <c r="B1" t="s">
+        <v>446</v>
+      </c>
+      <c r="C1" t="s">
+        <v>447</v>
+      </c>
+      <c r="D1" t="s">
+        <v>448</v>
+      </c>
+      <c r="E1" t="s">
+        <v>469</v>
+      </c>
+      <c r="F1" t="s">
+        <v>449</v>
+      </c>
+      <c r="G1" t="s">
+        <v>450</v>
+      </c>
+      <c r="H1" t="s">
+        <v>451</v>
+      </c>
+      <c r="I1" t="s">
+        <v>452</v>
+      </c>
+      <c r="J1" t="s">
+        <v>453</v>
+      </c>
+      <c r="K1" t="s">
+        <v>454</v>
+      </c>
+      <c r="L1" t="s">
+        <v>455</v>
+      </c>
+      <c r="M1" t="s">
+        <v>456</v>
+      </c>
+      <c r="N1" t="s">
+        <v>457</v>
+      </c>
+      <c r="O1" t="s">
+        <v>458</v>
+      </c>
+      <c r="P1" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>460</v>
+      </c>
+      <c r="B2" t="s">
+        <v>471</v>
+      </c>
+      <c r="C2" t="s">
+        <v>462</v>
+      </c>
+      <c r="D2" t="s">
+        <v>472</v>
+      </c>
+      <c r="E2" t="s">
+        <v>473</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>474</v>
+      </c>
+      <c r="G2" t="str">
+        <f>SUBSTITUTE(LOWER(H2)," ","")</f>
+        <v>firststage</v>
+      </c>
+      <c r="H2" t="s">
+        <v>475</v>
+      </c>
+      <c r="I2" t="str">
+        <f>LOWER(J2)</f>
+        <v>external</v>
+      </c>
+      <c r="J2" t="s">
+        <v>476</v>
+      </c>
+      <c r="K2" t="str">
+        <f>LOWER(L2)</f>
+        <v>right</v>
+      </c>
+      <c r="L2" t="s">
+        <v>185</v>
+      </c>
+      <c r="M2" t="s">
+        <v>477</v>
+      </c>
+      <c r="N2" t="str">
+        <f>LOWER(O2)</f>
+        <v>requested</v>
+      </c>
+      <c r="O2" t="s">
+        <v>207</v>
+      </c>
+      <c r="P2" t="s">
+        <v>478</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D695AEBB-372B-4AEC-8EA9-31363B2BEC69}">
+  <dimension ref="A1:K7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="21.26953125" customWidth="1"/>
+    <col min="11" max="11" width="37.08984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>480</v>
+      </c>
+      <c r="B1" t="s">
+        <v>481</v>
+      </c>
+      <c r="C1" t="s">
+        <v>482</v>
+      </c>
+      <c r="D1" t="s">
+        <v>483</v>
+      </c>
+      <c r="E1" t="s">
+        <v>484</v>
+      </c>
+      <c r="F1" t="s">
+        <v>485</v>
+      </c>
+      <c r="G1" t="s">
+        <v>486</v>
+      </c>
+      <c r="H1" t="s">
+        <v>487</v>
+      </c>
+      <c r="I1" t="s">
+        <v>488</v>
+      </c>
+      <c r="J1" t="s">
+        <v>489</v>
+      </c>
+      <c r="K1" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>491</v>
+      </c>
+      <c r="B2" t="s">
+        <v>492</v>
+      </c>
+      <c r="C2" t="s">
+        <v>493</v>
+      </c>
+      <c r="D2" t="s">
+        <v>494</v>
+      </c>
+      <c r="E2" t="s">
+        <v>495</v>
+      </c>
+      <c r="F2" t="s">
+        <v>496</v>
+      </c>
+      <c r="G2" t="s">
+        <v>497</v>
+      </c>
+      <c r="K2" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>499</v>
+      </c>
+      <c r="B3" t="s">
+        <v>500</v>
+      </c>
+      <c r="C3" t="s">
+        <v>501</v>
+      </c>
+      <c r="D3" t="s">
+        <v>100</v>
+      </c>
+      <c r="K3" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>503</v>
+      </c>
+      <c r="B4" t="s">
+        <v>504</v>
+      </c>
+      <c r="C4" t="s">
+        <v>505</v>
+      </c>
+      <c r="D4" t="s">
+        <v>506</v>
+      </c>
+      <c r="E4" t="s">
+        <v>507</v>
+      </c>
+      <c r="K4" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>509</v>
+      </c>
+      <c r="B5" t="s">
+        <v>510</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="D5" t="s">
+        <v>512</v>
+      </c>
+      <c r="E5" t="s">
+        <v>513</v>
+      </c>
+      <c r="F5" t="s">
+        <v>510</v>
+      </c>
+      <c r="G5" t="s">
+        <v>511</v>
+      </c>
+      <c r="H5" t="s">
+        <v>512</v>
+      </c>
+      <c r="I5" t="s">
+        <v>100</v>
+      </c>
+      <c r="J5" t="s">
+        <v>100</v>
+      </c>
+      <c r="K5" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C7" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A6010D5-47E1-495B-AA2A-B893D5A1F055}">
+  <dimension ref="A1:N5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.26953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="36.90625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.08984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>480</v>
+      </c>
+      <c r="B1" t="s">
+        <v>481</v>
+      </c>
+      <c r="C1" t="s">
+        <v>482</v>
+      </c>
+      <c r="D1" t="s">
+        <v>483</v>
+      </c>
+      <c r="E1" t="s">
+        <v>484</v>
+      </c>
+      <c r="F1" t="s">
+        <v>485</v>
+      </c>
+      <c r="G1" t="s">
+        <v>486</v>
+      </c>
+      <c r="H1" t="s">
+        <v>487</v>
+      </c>
+      <c r="I1" t="s">
+        <v>488</v>
+      </c>
+      <c r="J1" t="s">
+        <v>489</v>
+      </c>
+      <c r="K1" t="s">
+        <v>490</v>
+      </c>
+      <c r="L1" t="s">
+        <v>515</v>
+      </c>
+      <c r="M1" t="s">
+        <v>516</v>
+      </c>
+      <c r="N1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>491</v>
+      </c>
+      <c r="B2" t="s">
+        <v>517</v>
+      </c>
+      <c r="C2" t="s">
+        <v>518</v>
+      </c>
+      <c r="D2" t="s">
+        <v>519</v>
+      </c>
+      <c r="E2" t="s">
+        <v>520</v>
+      </c>
+      <c r="F2" t="s">
+        <v>521</v>
+      </c>
+      <c r="G2" t="s">
+        <v>522</v>
+      </c>
+      <c r="K2" t="s">
+        <v>523</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="N2" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>499</v>
+      </c>
+      <c r="B3" t="s">
+        <v>526</v>
+      </c>
+      <c r="C3" t="s">
+        <v>527</v>
+      </c>
+      <c r="D3" t="s">
+        <v>60</v>
+      </c>
+      <c r="K3" t="s">
+        <v>528</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="N3" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>503</v>
+      </c>
+      <c r="B4" t="s">
+        <v>529</v>
+      </c>
+      <c r="C4" t="s">
+        <v>530</v>
+      </c>
+      <c r="D4" t="s">
+        <v>531</v>
+      </c>
+      <c r="E4" t="s">
+        <v>532</v>
+      </c>
+      <c r="K4" t="s">
+        <v>533</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="N4" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>509</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="C5" t="s">
+        <v>512</v>
+      </c>
+      <c r="D5" t="s">
+        <v>513</v>
+      </c>
+      <c r="E5" t="s">
+        <v>510</v>
+      </c>
+      <c r="F5" t="s">
+        <v>511</v>
+      </c>
+      <c r="G5" t="s">
+        <v>512</v>
+      </c>
+      <c r="H5" t="s">
+        <v>510</v>
+      </c>
+      <c r="I5" t="s">
+        <v>60</v>
+      </c>
+      <c r="J5" t="s">
+        <v>60</v>
+      </c>
+      <c r="K5" t="s">
+        <v>534</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="M5" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="N5" t="s">
+        <v>525</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23837C59-F13D-4C7B-A343-BB4EFCC5792C}">
+  <dimension ref="A1:U4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="17.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="17.6328125" customWidth="1"/>
+    <col min="8" max="8" width="24" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="32.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.6328125" customWidth="1"/>
+    <col min="11" max="11" width="26" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="23.7265625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.26953125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="23.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="25.453125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="23.1796875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="27.81640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="21.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" t="s">
+        <v>540</v>
+      </c>
+      <c r="C1" t="s">
+        <v>541</v>
+      </c>
+      <c r="D1" t="s">
+        <v>542</v>
+      </c>
+      <c r="E1" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1" t="s">
+        <v>544</v>
+      </c>
+      <c r="G1" t="s">
+        <v>584</v>
+      </c>
+      <c r="H1" t="s">
+        <v>585</v>
+      </c>
+      <c r="I1" t="s">
+        <v>586</v>
+      </c>
+      <c r="J1" t="s">
+        <v>587</v>
+      </c>
+      <c r="K1" t="s">
+        <v>588</v>
+      </c>
+      <c r="L1" t="s">
+        <v>589</v>
+      </c>
+      <c r="M1" t="s">
+        <v>590</v>
+      </c>
+      <c r="N1" t="s">
+        <v>591</v>
+      </c>
+      <c r="O1" t="s">
+        <v>545</v>
+      </c>
+      <c r="P1" t="s">
+        <v>592</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>593</v>
+      </c>
+      <c r="R1" t="s">
+        <v>594</v>
+      </c>
+      <c r="S1" t="s">
+        <v>595</v>
+      </c>
+      <c r="T1" t="s">
+        <v>551</v>
+      </c>
+      <c r="U1" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>546</v>
+      </c>
+      <c r="B2" t="s">
+        <v>572</v>
+      </c>
+      <c r="C2" t="s">
+        <v>573</v>
+      </c>
+      <c r="D2" t="s">
+        <v>574</v>
+      </c>
+      <c r="E2" t="s">
+        <v>575</v>
+      </c>
+      <c r="F2" t="s">
+        <v>576</v>
+      </c>
+      <c r="G2" t="s">
+        <v>577</v>
+      </c>
+      <c r="H2" t="s">
+        <v>600</v>
+      </c>
+      <c r="I2" t="s">
+        <v>578</v>
+      </c>
+      <c r="J2" t="s">
+        <v>579</v>
+      </c>
+      <c r="K2" t="s">
+        <v>580</v>
+      </c>
+      <c r="L2" t="s">
+        <v>581</v>
+      </c>
+      <c r="M2" t="s">
+        <v>582</v>
+      </c>
+      <c r="N2" t="s">
+        <v>583</v>
+      </c>
+      <c r="P2" t="s">
+        <v>596</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>597</v>
+      </c>
+      <c r="R2" t="s">
+        <v>598</v>
+      </c>
+      <c r="S2" t="s">
+        <v>599</v>
+      </c>
+      <c r="U2" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>553</v>
+      </c>
+      <c r="B3" t="s">
+        <v>549</v>
+      </c>
+      <c r="C3" t="s">
+        <v>550</v>
+      </c>
+      <c r="D3" t="s">
+        <v>319</v>
+      </c>
+      <c r="O3" t="s">
+        <v>548</v>
+      </c>
+      <c r="T3" t="s">
+        <v>552</v>
+      </c>
+      <c r="U3" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>564</v>
+      </c>
+      <c r="O4" t="s">
+        <v>565</v>
+      </c>
+      <c r="T4" t="s">
+        <v>567</v>
+      </c>
+      <c r="U4" t="s">
+        <v>566</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52CEE698-ED81-42DF-AF70-0D9AAC45D1CA}">
+  <dimension ref="A1:X5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="14.54296875" customWidth="1"/>
+    <col min="2" max="3" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="31.1796875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="21.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="22.08984375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="18" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" t="s">
+        <v>540</v>
+      </c>
+      <c r="C1" t="s">
+        <v>541</v>
+      </c>
+      <c r="D1" t="s">
+        <v>542</v>
+      </c>
+      <c r="E1" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1" t="s">
+        <v>544</v>
+      </c>
+      <c r="G1" t="s">
+        <v>584</v>
+      </c>
+      <c r="H1" t="s">
+        <v>585</v>
+      </c>
+      <c r="I1" t="s">
+        <v>586</v>
+      </c>
+      <c r="J1" t="s">
+        <v>587</v>
+      </c>
+      <c r="K1" t="s">
+        <v>588</v>
+      </c>
+      <c r="L1" t="s">
+        <v>589</v>
+      </c>
+      <c r="M1" t="s">
+        <v>590</v>
+      </c>
+      <c r="N1" t="s">
+        <v>591</v>
+      </c>
+      <c r="O1" t="s">
+        <v>545</v>
+      </c>
+      <c r="P1" t="s">
+        <v>592</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>593</v>
+      </c>
+      <c r="R1" t="s">
+        <v>594</v>
+      </c>
+      <c r="S1" t="s">
+        <v>595</v>
+      </c>
+      <c r="T1" t="s">
+        <v>554</v>
+      </c>
+      <c r="U1" t="s">
+        <v>133</v>
+      </c>
+      <c r="V1" t="s">
+        <v>556</v>
+      </c>
+      <c r="W1" t="s">
+        <v>557</v>
+      </c>
+      <c r="X1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>546</v>
+      </c>
+      <c r="B2" t="s">
+        <v>576</v>
+      </c>
+      <c r="C2" t="s">
+        <v>577</v>
+      </c>
+      <c r="D2" t="s">
+        <v>605</v>
+      </c>
+      <c r="E2" t="s">
+        <v>606</v>
+      </c>
+      <c r="F2" t="s">
+        <v>572</v>
+      </c>
+      <c r="G2" t="s">
+        <v>573</v>
+      </c>
+      <c r="H2" t="s">
+        <v>607</v>
+      </c>
+      <c r="I2" t="s">
+        <v>581</v>
+      </c>
+      <c r="J2" t="s">
+        <v>582</v>
+      </c>
+      <c r="K2" t="s">
+        <v>608</v>
+      </c>
+      <c r="L2" t="s">
+        <v>578</v>
+      </c>
+      <c r="M2" t="s">
+        <v>579</v>
+      </c>
+      <c r="N2" t="s">
+        <v>609</v>
+      </c>
+      <c r="P2" t="s">
+        <v>601</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>602</v>
+      </c>
+      <c r="R2" t="s">
+        <v>603</v>
+      </c>
+      <c r="S2" t="s">
+        <v>604</v>
+      </c>
+      <c r="T2" t="s">
+        <v>546</v>
+      </c>
+      <c r="U2" s="6" t="s">
+        <v>555</v>
+      </c>
+      <c r="V2" s="6" t="s">
+        <v>555</v>
+      </c>
+      <c r="W2" s="6" t="s">
+        <v>555</v>
+      </c>
+      <c r="X2" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>553</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>559</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>560</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>561</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>562</v>
+      </c>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" t="s">
+        <v>563</v>
+      </c>
+      <c r="T3" t="s">
+        <v>547</v>
+      </c>
+      <c r="V3" s="6" t="s">
+        <v>555</v>
+      </c>
+      <c r="W3" s="6" t="s">
+        <v>555</v>
+      </c>
+      <c r="X3" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>564</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>568</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>569</v>
+      </c>
+      <c r="O4" t="s">
+        <v>570</v>
+      </c>
+      <c r="T4" t="s">
+        <v>566</v>
+      </c>
+      <c r="V4" s="6" t="s">
+        <v>571</v>
+      </c>
+      <c r="W4" s="6" t="s">
+        <v>571</v>
+      </c>
+      <c r="X4" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="V5" s="6"/>
+      <c r="W5" s="6"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3310FF1D-4559-4E35-BB7B-0285AF82C887}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
   </cols>
@@ -5869,19 +7570,19 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82EC7FC3-A185-46F7-A2D4-55C9E247ADD9}">
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="23.85546875" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" customWidth="1"/>
-    <col min="4" max="4" width="22.28515625" customWidth="1"/>
-    <col min="5" max="5" width="17.42578125" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" customWidth="1"/>
-    <col min="7" max="7" width="17.5703125" customWidth="1"/>
-    <col min="8" max="8" width="16.5703125" customWidth="1"/>
-    <col min="9" max="9" width="26.85546875" customWidth="1"/>
+    <col min="1" max="2" width="23.81640625" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" customWidth="1"/>
+    <col min="4" max="4" width="22.26953125" customWidth="1"/>
+    <col min="5" max="5" width="17.453125" customWidth="1"/>
+    <col min="6" max="6" width="15.1796875" customWidth="1"/>
+    <col min="7" max="7" width="17.54296875" customWidth="1"/>
+    <col min="8" max="8" width="16.54296875" customWidth="1"/>
+    <col min="9" max="9" width="26.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -5910,7 +7611,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>200</v>
       </c>
@@ -5947,18 +7648,18 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{538BA7B8-E3A5-4977-A6D8-AD18062987D5}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" customWidth="1"/>
-    <col min="5" max="5" width="16.42578125" customWidth="1"/>
-    <col min="6" max="6" width="15.28515625" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.453125" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" customWidth="1"/>
+    <col min="4" max="4" width="14.453125" customWidth="1"/>
+    <col min="5" max="5" width="16.453125" customWidth="1"/>
+    <col min="6" max="6" width="15.26953125" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -5978,7 +7679,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>200</v>
       </c>
@@ -6004,6 +7705,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="563c2453-77f6-4899-a3ec-7eb6553b4f66">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="c9416fa7-6169-4354-a691-3cfdebf72cd6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100957D2DE5FA4F58469907EC3226CC7D98" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="090753d51dfd09a1119d54c5de179dfc">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="563c2453-77f6-4899-a3ec-7eb6553b4f66" xmlns:ns3="c9416fa7-6169-4354-a691-3cfdebf72cd6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9c8570d9b0f0a7b9a0c34f8b658bbfee" ns2:_="" ns3:_="">
     <xsd:import namespace="563c2453-77f6-4899-a3ec-7eb6553b4f66"/>
@@ -6258,27 +7979,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="563c2453-77f6-4899-a3ec-7eb6553b4f66">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="c9416fa7-6169-4354-a691-3cfdebf72cd6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE0B556D-2173-4F7C-9F53-AE9A9D15CB9C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="563c2453-77f6-4899-a3ec-7eb6553b4f66"/>
+    <ds:schemaRef ds:uri="c9416fa7-6169-4354-a691-3cfdebf72cd6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{101DBEFA-2EFF-47B2-92EB-3E72B43EE2A6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1EC2FBF-A56D-40AC-8C09-CB1DCD191DD4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6295,23 +8015,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE0B556D-2173-4F7C-9F53-AE9A9D15CB9C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="563c2453-77f6-4899-a3ec-7eb6553b4f66"/>
-    <ds:schemaRef ds:uri="c9416fa7-6169-4354-a691-3cfdebf72cd6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{101DBEFA-2EFF-47B2-92EB-3E72B43EE2A6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Added Patient View and Patient Consent category changes
</commit_message>
<xml_diff>
--- a/ExcelFiles/PatientSummary.xlsx
+++ b/ExcelFiles/PatientSummary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Riomed\Cellma4ClinicalAuto\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93063035-C3AC-415E-8615-134F10C01031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE322496-E374-4DE8-9399-6A626D1618CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-21600" windowWidth="19410" windowHeight="20985" firstSheet="62" activeTab="67" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" firstSheet="63" activeTab="69" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loginDetails" sheetId="2" r:id="rId1"/>
@@ -81,6 +81,8 @@
     <sheet name="EditTest" sheetId="67" r:id="rId66"/>
     <sheet name="AddTool" sheetId="68" r:id="rId67"/>
     <sheet name="EditTool" sheetId="69" r:id="rId68"/>
+    <sheet name="AddPatientConsent" sheetId="70" r:id="rId69"/>
+    <sheet name="EditPatientConsent" sheetId="71" r:id="rId70"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -103,7 +105,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1228" uniqueCount="610">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1301" uniqueCount="658">
   <si>
     <t>username</t>
   </si>
@@ -1933,6 +1935,150 @@
   </si>
   <si>
     <t>Reliability Aided Soundfield Edited</t>
+  </si>
+  <si>
+    <t>pac_consent_given_by</t>
+  </si>
+  <si>
+    <t>pac_consent_type</t>
+  </si>
+  <si>
+    <t>pac_consent_status</t>
+  </si>
+  <si>
+    <t>pac_consent_start</t>
+  </si>
+  <si>
+    <t>pac_consent_end</t>
+  </si>
+  <si>
+    <t>pac_consent_file_path</t>
+  </si>
+  <si>
+    <t>pac_consent_file</t>
+  </si>
+  <si>
+    <t>pac_consent_file_type</t>
+  </si>
+  <si>
+    <t>pac_notes</t>
+  </si>
+  <si>
+    <t>pac_special_requirement</t>
+  </si>
+  <si>
+    <t>pac_medical_term</t>
+  </si>
+  <si>
+    <t>pac_intended_benefits</t>
+  </si>
+  <si>
+    <t>pac_frequent_risks</t>
+  </si>
+  <si>
+    <t>pac_blood_transfusion</t>
+  </si>
+  <si>
+    <t>pac_procedures</t>
+  </si>
+  <si>
+    <t>pac_risks</t>
+  </si>
+  <si>
+    <t>Wednesday Tester</t>
+  </si>
+  <si>
+    <t>Contact by Email</t>
+  </si>
+  <si>
+    <t>Given</t>
+  </si>
+  <si>
+    <t>\consent\4\788397</t>
+  </si>
+  <si>
+    <t>pac_4771_dummy.pdf</t>
+  </si>
+  <si>
+    <t>pdf</t>
+  </si>
+  <si>
+    <t>Data entry test.</t>
+  </si>
+  <si>
+    <t>This is a special requirement</t>
+  </si>
+  <si>
+    <t>Brief explanation of term used</t>
+  </si>
+  <si>
+    <t>This is an intended benefit</t>
+  </si>
+  <si>
+    <t>This is a risk that occurs often</t>
+  </si>
+  <si>
+    <t>Details for blood transfusion</t>
+  </si>
+  <si>
+    <t>Details of procedure</t>
+  </si>
+  <si>
+    <t>These are risks</t>
+  </si>
+  <si>
+    <t>medi_form</t>
+  </si>
+  <si>
+    <t>tablet</t>
+  </si>
+  <si>
+    <t>01/04/2025</t>
+  </si>
+  <si>
+    <t>pac_consent_details_json</t>
+  </si>
+  <si>
+    <t>Record edit test</t>
+  </si>
+  <si>
+    <t>Withdrawn</t>
+  </si>
+  <si>
+    <t>Edited requirement</t>
+  </si>
+  <si>
+    <t>No term explanation needed</t>
+  </si>
+  <si>
+    <t>Benefit of knowledge</t>
+  </si>
+  <si>
+    <t>No risks</t>
+  </si>
+  <si>
+    <t>Blood transfusion was done</t>
+  </si>
+  <si>
+    <t>No procedure</t>
+  </si>
+  <si>
+    <t>Risk of boredom</t>
+  </si>
+  <si>
+    <t>pac_withdraw_date</t>
+  </si>
+  <si>
+    <t>01/05/2025</t>
+  </si>
+  <si>
+    <t>{"patientDetails":{"patSurname":"Riomedtest","patFirstName":"AkaliA","patDateOfBirth":"08/09/2024","patGender":"M","patNhsNumber":"","patPid":"","specialRequirements":"This is a special requirement","proposedProcedures":{},"briefExplanationMedicalTerm":"Brief explanation of term used"},"statementOfHealthProfessional":{"explainedIntendedBenefits":"This is an intended benefit","significantUnavoidableRisks":"This is a risk that occurs often","extraProcedures":{"bloodTransfusion":true,"details":"Details for blood transfusion","proceduresChecked":true,"otherProcedures":[{},{"details":"Details of procedure"}]},"providedInformation":true,"details":"These are risks","involvedProcedureDetails":{"generalAnaesthesia":false,"localAnaesthesia":false,"sedation":false,"responsibleHealthProfessional":{"name":"","jobTitle":"","registrationNumber":"","signature":""},"healthProfessionalName":"","jobTitle":"","date":"18/06/2025"}},"statementOfInterpreter":{"signature":"","interpreterName":"","date":"18/06/2025"},"statementOfParent":{"details":"","removelOfTissueOrBloodDuringOperation":"Yes","forResearchInConnectionWithDisorders":"Yes","forScientificOrMedicalInformation":"Yes","parentDetails":{"patientSignature":"","patientName":"AkaliA Riomedtest","date":null},"witnessDetails":{"patientSignature":"","patientName":"","date":null}},"confirmationOfConsent":{"healthProfessional":{"signature":"","name":"","jobTitle":"","date":null},"parent":{"signature":"","name":"AkaliA Riomedtest","date":null}},"withdrawalOfConsentDetails":{"patientName":"AkaliA Riomedtest","date":null}}</t>
+  </si>
+  <si>
+    <t>{"patientDetails":{"patSurname":"Riomedtest","patFirstName":"AkaliA","patDateOfBirth":"08/09/2024","patGender":"M","patNhsNumber":"","patPid":"","specialRequirements":"Edited requirement","proposedProcedures":{},"briefExplanationMedicalTerm":"No term explanation needed"},"statementOfHealthProfessional":{"explainedIntendedBenefits":"Benefit of knowledge","significantUnavoidableRisks":"No risks","extraProcedures":{"bloodTransfusion":false,"details":"Blood transfusion was done","proceduresChecked":true,"otherProcedures":[{},{"details":"No procedure"}]},"providedInformation":true,"details":"Risk of boredom","involvedProcedureDetails":{"generalAnaesthesia":false,"localAnaesthesia":false,"sedation":false,"responsibleHealthProfessional":{"name":"","jobTitle":"","registrationNumber":"","signature":""},"healthProfessionalName":"","jobTitle":"","date":"18/06/2025"}},"statementOfInterpreter":{"signature":"","interpreterName":"","date":"18/06/2025"},"statementOfParent":{"details":"","removelOfTissueOrBloodDuringOperation":"Yes","forResearchInConnectionWithDisorders":"Yes","forScientificOrMedicalInformation":"Yes","parentDetails":{"patientSignature":"","patientName":"AkaliA Riomedtest","date":null},"witnessDetails":{"patientSignature":"","patientName":"","date":null}},"confirmationOfConsent":{"healthProfessional":{"signature":"","name":"","jobTitle":"","date":null},"parent":{"signature":"","name":"AkaliA Riomedtest","date":null}},"withdrawalOfConsentDetails":{"withdrawnConsent":true,"patientName":"AkaliA Riomedtest","date":"18/06/2025"}}</t>
+  </si>
+  <si>
+    <t>pac_consent_status_input</t>
   </si>
 </sst>
 </file>
@@ -3446,7 +3592,7 @@
       </c>
       <c r="D2" s="7" t="str">
         <f ca="1">TEXT(TODAY(), "DD/MM/YYYY")</f>
-        <v>17/06/2025</v>
+        <v>18/06/2025</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>198</v>
@@ -3520,7 +3666,7 @@
       </c>
       <c r="D2" s="7" t="str">
         <f ca="1">TEXT(TODAY(), "DD/MM/YYYY")</f>
-        <v>17/06/2025</v>
+        <v>18/06/2025</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>199</v>
@@ -3751,7 +3897,7 @@
       </c>
       <c r="C2" s="7">
         <f ca="1">TODAY()</f>
-        <v>45825</v>
+        <v>45826</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>103</v>
@@ -4502,44 +4648,45 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DD9439C-0973-45AC-88BC-21584AF7E144}">
-  <dimension ref="A1:AG2"/>
+  <dimension ref="A1:AH2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="40.6328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.90625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.6328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.08984375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.1796875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="23.81640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="21.26953125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="27.90625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="32.26953125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="25.7265625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="23.453125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="21.26953125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="23.453125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="21.90625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.36328125" customWidth="1"/>
+    <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="23.81640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="21.26953125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="27.90625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="32.26953125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="25.7265625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="23.453125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="21.26953125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="23.453125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="21.90625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -4550,97 +4697,100 @@
         <v>69</v>
       </c>
       <c r="D1" t="s">
+        <v>640</v>
+      </c>
+      <c r="E1" t="s">
         <v>70</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>72</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>81</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>74</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>101</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>75</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>76</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>94</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>95</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>79</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>80</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>97</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>179</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>537</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>90</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>92</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>99</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>96</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>114</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>106</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>104</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>107</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>108</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>110</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>107</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AD1" t="s">
         <v>112</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AE1" t="s">
         <v>127</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AF1" t="s">
         <v>181</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AG1" t="s">
         <v>202</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AH1" t="s">
         <v>535</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>223</v>
       </c>
@@ -4650,88 +4800,91 @@
       <c r="C2" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="E2" t="s">
         <v>71</v>
-      </c>
-      <c r="E2" t="s">
-        <v>73</v>
       </c>
       <c r="F2" t="s">
         <v>73</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" t="s">
+        <v>73</v>
+      </c>
+      <c r="H2" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="I2" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="J2" s="7" t="s">
         <v>435</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="K2" s="7" t="s">
         <v>436</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>177</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>83</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>98</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>180</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>85</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>91</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>93</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
         <v>100</v>
       </c>
-      <c r="U2" s="6" t="s">
+      <c r="V2" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="V2" s="6" t="s">
+      <c r="W2" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="W2" t="s">
+      <c r="X2" t="s">
         <v>102</v>
       </c>
-      <c r="X2" t="s">
+      <c r="Y2" t="s">
         <v>105</v>
       </c>
-      <c r="Y2" s="6" t="s">
+      <c r="Z2" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="Z2" t="s">
+      <c r="AA2" t="s">
         <v>109</v>
       </c>
-      <c r="AA2" s="6" t="s">
+      <c r="AB2" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="AB2">
+      <c r="AC2">
         <v>5</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AD2" t="s">
         <v>111</v>
       </c>
-      <c r="AD2" t="s">
+      <c r="AE2" t="s">
         <v>176</v>
       </c>
-      <c r="AE2" t="s">
+      <c r="AF2" t="s">
         <v>182</v>
       </c>
-      <c r="AF2" s="9" t="s">
+      <c r="AG2" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="AG2" t="s">
+      <c r="AH2" t="s">
         <v>536</v>
       </c>
     </row>
@@ -6286,7 +6439,7 @@
       </c>
       <c r="B2" s="8" t="str">
         <f ca="1">TEXT(TODAY(), "DD/MM/YYYY")</f>
-        <v>17/06/2025</v>
+        <v>18/06/2025</v>
       </c>
       <c r="C2" t="s">
         <v>417</v>
@@ -7555,6 +7708,141 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8527E2DD-D099-43B2-BA92-EA00DEE08B55}">
+  <dimension ref="A1:Q2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="24.6328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="26.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="25.6328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="24.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.90625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="255.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>610</v>
+      </c>
+      <c r="B1" t="s">
+        <v>611</v>
+      </c>
+      <c r="C1" t="s">
+        <v>612</v>
+      </c>
+      <c r="D1" t="s">
+        <v>613</v>
+      </c>
+      <c r="E1" t="s">
+        <v>614</v>
+      </c>
+      <c r="F1" t="s">
+        <v>615</v>
+      </c>
+      <c r="G1" t="s">
+        <v>616</v>
+      </c>
+      <c r="H1" t="s">
+        <v>617</v>
+      </c>
+      <c r="I1" t="s">
+        <v>618</v>
+      </c>
+      <c r="J1" t="s">
+        <v>619</v>
+      </c>
+      <c r="K1" t="s">
+        <v>620</v>
+      </c>
+      <c r="L1" t="s">
+        <v>621</v>
+      </c>
+      <c r="M1" t="s">
+        <v>622</v>
+      </c>
+      <c r="N1" t="s">
+        <v>623</v>
+      </c>
+      <c r="O1" t="s">
+        <v>624</v>
+      </c>
+      <c r="P1" t="s">
+        <v>625</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>626</v>
+      </c>
+      <c r="B2" t="s">
+        <v>627</v>
+      </c>
+      <c r="C2" t="s">
+        <v>628</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>654</v>
+      </c>
+      <c r="F2" t="s">
+        <v>629</v>
+      </c>
+      <c r="G2" t="s">
+        <v>630</v>
+      </c>
+      <c r="H2" t="s">
+        <v>631</v>
+      </c>
+      <c r="I2" t="s">
+        <v>632</v>
+      </c>
+      <c r="J2" t="s">
+        <v>633</v>
+      </c>
+      <c r="K2" t="s">
+        <v>634</v>
+      </c>
+      <c r="L2" t="s">
+        <v>635</v>
+      </c>
+      <c r="M2" t="s">
+        <v>636</v>
+      </c>
+      <c r="N2" t="s">
+        <v>637</v>
+      </c>
+      <c r="O2" t="s">
+        <v>638</v>
+      </c>
+      <c r="P2" t="s">
+        <v>639</v>
+      </c>
+      <c r="Q2" s="11" t="s">
+        <v>655</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3310FF1D-4559-4E35-BB7B-0285AF82C887}">
   <dimension ref="A1"/>
@@ -7564,6 +7852,155 @@
   </cols>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EDC6A1B-AAB3-467B-B35D-67887A5D3127}">
+  <dimension ref="A1:S2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.453125" customWidth="1"/>
+    <col min="5" max="5" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.08984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.90625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.08984375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="24.26953125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>610</v>
+      </c>
+      <c r="B1" t="s">
+        <v>611</v>
+      </c>
+      <c r="C1" t="s">
+        <v>657</v>
+      </c>
+      <c r="D1" t="s">
+        <v>612</v>
+      </c>
+      <c r="E1" t="s">
+        <v>613</v>
+      </c>
+      <c r="F1" t="s">
+        <v>614</v>
+      </c>
+      <c r="G1" t="s">
+        <v>653</v>
+      </c>
+      <c r="H1" t="s">
+        <v>615</v>
+      </c>
+      <c r="I1" t="s">
+        <v>616</v>
+      </c>
+      <c r="J1" t="s">
+        <v>617</v>
+      </c>
+      <c r="K1" t="s">
+        <v>618</v>
+      </c>
+      <c r="L1" t="s">
+        <v>619</v>
+      </c>
+      <c r="M1" t="s">
+        <v>620</v>
+      </c>
+      <c r="N1" t="s">
+        <v>621</v>
+      </c>
+      <c r="O1" t="s">
+        <v>622</v>
+      </c>
+      <c r="P1" t="s">
+        <v>623</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>624</v>
+      </c>
+      <c r="R1" t="s">
+        <v>625</v>
+      </c>
+      <c r="S1" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>626</v>
+      </c>
+      <c r="B2" t="s">
+        <v>627</v>
+      </c>
+      <c r="C2" t="s">
+        <v>645</v>
+      </c>
+      <c r="D2" t="str">
+        <f>LOWER(C2)</f>
+        <v>withdrawn</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>436</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>436</v>
+      </c>
+      <c r="H2" t="s">
+        <v>629</v>
+      </c>
+      <c r="I2" t="s">
+        <v>630</v>
+      </c>
+      <c r="J2" t="s">
+        <v>631</v>
+      </c>
+      <c r="K2" t="s">
+        <v>644</v>
+      </c>
+      <c r="L2" t="s">
+        <v>646</v>
+      </c>
+      <c r="M2" t="s">
+        <v>647</v>
+      </c>
+      <c r="N2" t="s">
+        <v>648</v>
+      </c>
+      <c r="O2" t="s">
+        <v>649</v>
+      </c>
+      <c r="P2" t="s">
+        <v>650</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>651</v>
+      </c>
+      <c r="R2" t="s">
+        <v>652</v>
+      </c>
+      <c r="S2" s="11" t="s">
+        <v>656</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>